<commit_message>
Fixed windows regressions and prepped for Mac     testing.
Added a pre commit hook to create an xlsx version
    of the template.
</commit_message>
<xml_diff>
--- a/src/xleda/xleda_template.xlsx
+++ b/src/xleda/xleda_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{136AFA62-E6A1-4F9C-84A0-32F91298B43C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BAF7F93-214C-46AF-8F30-A790E939C118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="1812" windowWidth="10980" windowHeight="8880" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Field Analysis" sheetId="25" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated examples, completed tests on Windows
</commit_message>
<xml_diff>
--- a/src/xleda/xleda_template.xlsx
+++ b/src/xleda/xleda_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrivers/Python/xleda/src/xleda/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B2DBF8E-069E-6E4E-9D38-77619E37DCA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF4A5511-2517-4497-9789-9637F3524CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19480" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Field Analysis" sheetId="25" r:id="rId1"/>
@@ -100,7 +100,7 @@
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -116,6 +116,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1379,74 +1382,41 @@
   <dxfs count="88">
     <dxf>
       <font>
-        <color theme="0"/>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1" tint="0.79998168889431442"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FF1EAC1D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF1EAC1D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="&quot;List names must be unique&quot;"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1474,16 +1444,296 @@
       </fill>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </left>
-        <right/>
+        <left/>
+        <right style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </right>
         <top style="thin">
           <color theme="1" tint="-0.499984740745262"/>
         </top>
         <bottom/>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1" tint="0.39997558519241921"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1" tint="0.39997558519241921"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1" tint="0.39997558519241921"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1" tint="0.39997558519241921"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FF1D1D1D"/>
+        </left>
+        <top style="thin">
+          <color rgb="FF1D1D1D"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1" tint="0.39997558519241921"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1" tint="0.79998168889431442"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0%"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <i/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1" tint="0.79998168889431442"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="#,##0.0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </left>
+        <right style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </right>
+        <top style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </top>
+        <bottom style="thin">
+          <color theme="1" tint="-0.499984740745262"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1506,324 +1756,6 @@
       <numFmt numFmtId="3" formatCode="#,##0"/>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color rgb="FF1D1D1D"/>
-        </left>
-        <top style="thin">
-          <color rgb="FF1D1D1D"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.79998168889431442"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0%"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.79998168889431442"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="#,##0.0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.79998168889431442"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -2871,6 +2803,77 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF1EAC1D"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="&quot;List names must be unique&quot;"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF1EAC1D"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3100,7 +3103,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B0C8B3AD-C6E3-47A6-946E-3DF35EDAC621}" name="pvt_Pivot" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showError="1" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B0C8B3AD-C6E3-47A6-946E-3DF35EDAC621}" name="pvt_Pivot" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" showError="1" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="C9:E10" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="4">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -3131,16 +3134,16 @@
     <dataField name="% of Records" fld="2" subtotal="count" showDataAs="percentOfTotal" baseField="0" baseItem="2" numFmtId="10"/>
   </dataFields>
   <formats count="19">
-    <format dxfId="48">
+    <format dxfId="41">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="47">
+    <format dxfId="40">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="46">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="45">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -3150,10 +3153,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="37">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="43">
+    <format dxfId="36">
       <pivotArea dataOnly="0" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3162,7 +3165,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="42">
+    <format dxfId="35">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3171,7 +3174,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="34">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3180,16 +3183,16 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="40">
+    <format dxfId="33">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="39">
+    <format dxfId="32">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="31">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="37">
+    <format dxfId="30">
       <pivotArea dataOnly="0" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -3199,7 +3202,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="36">
+    <format dxfId="29">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -3208,7 +3211,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="35">
+    <format dxfId="28">
       <pivotArea dataOnly="0" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3217,13 +3220,13 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="34">
+    <format dxfId="27">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="26">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="25">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -3232,7 +3235,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="24">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="3">
@@ -3243,7 +3246,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="23">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="3">
@@ -3356,91 +3359,91 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DB1D1E60-5E37-456A-AD85-0649D531840E}" name="tbl_SourceData" displayName="tbl_SourceData" ref="D79:G81" totalsRowShown="0" dataDxfId="82" headerRowCellStyle="DarkHeader" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DB1D1E60-5E37-456A-AD85-0649D531840E}" name="tbl_SourceData" displayName="tbl_SourceData" ref="D79:G81" totalsRowShown="0" dataDxfId="75" headerRowCellStyle="DarkHeader" dataCellStyle="Normal">
   <autoFilter ref="D79:G81" xr:uid="{DB1D1E60-5E37-456A-AD85-0649D531840E}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{57EDF41E-F06D-4819-BADE-3D62DE46F06C}" name="Record List" dataDxfId="81" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{CF70C9CE-83FE-40FA-8089-C68B39CF665A}" name="DarkHeader" dataDxfId="80" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{B8654690-502A-4FAF-9205-0118DABCB954}" name="HasBlank" dataDxfId="79" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{5A5BA001-2F93-4E62-880C-C4E8BDB17EEB}" name="FormatRange" dataDxfId="78" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{57EDF41E-F06D-4819-BADE-3D62DE46F06C}" name="Record List" dataDxfId="74" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{CF70C9CE-83FE-40FA-8089-C68B39CF665A}" name="DarkHeader" dataDxfId="73" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{B8654690-502A-4FAF-9205-0118DABCB954}" name="HasBlank" dataDxfId="72" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{5A5BA001-2F93-4E62-880C-C4E8BDB17EEB}" name="FormatRange" dataDxfId="71" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{034D1C74-BE18-490E-B396-097D407DA97D}" name="tbl_Overview" displayName="tbl_Overview" ref="B11:AA12" totalsRowShown="0" headerRowDxfId="77" dataDxfId="75" headerRowBorderDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{034D1C74-BE18-490E-B396-097D407DA97D}" name="tbl_Overview" displayName="tbl_Overview" ref="B11:AA12" totalsRowShown="0" headerRowDxfId="70" dataDxfId="68" headerRowBorderDxfId="69">
   <autoFilter ref="B11:AA12" xr:uid="{034D1C74-BE18-490E-B396-097D407DA97D}"/>
   <tableColumns count="26">
-    <tableColumn id="1" xr3:uid="{010A8E62-502A-4B19-B37A-BF59E03A068A}" name="Field" dataDxfId="74"/>
-    <tableColumn id="2" xr3:uid="{AD236665-EC7C-404F-8915-AD7CD5510D0F}" name="Definition" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{B78AB378-5727-433E-AB9C-BB970FC42B31}" name="Field Notes" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{EF15AE67-FE31-471E-840E-8104B878A3E8}" name="Data type" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{5006D683-9D12-4B97-9EF2-6D41AF6E0B35}" name="Distinct %" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{3AFB42F8-9976-44FF-9239-74914D5BE035}" name="Missing %" dataDxfId="69"/>
-    <tableColumn id="7" xr3:uid="{4BA41102-DB06-4180-9754-C88722FE82BD}" name="Memory Usage %" dataDxfId="68"/>
-    <tableColumn id="8" xr3:uid="{D22319BD-3A80-40F3-84FC-A6D1627B2F29}" name="Memory Usage" dataDxfId="67"/>
-    <tableColumn id="9" xr3:uid="{77FAEE19-B6C7-4056-8EF3-5EB877C820C4}" name="Distinct" dataDxfId="66"/>
-    <tableColumn id="10" xr3:uid="{54FF47BF-594E-417B-9028-64A4DFE4D389}" name="Count" dataDxfId="65"/>
-    <tableColumn id="11" xr3:uid="{54E587FE-36DC-4522-91DC-8B81B386217B}" name="Count %" dataDxfId="64"/>
-    <tableColumn id="12" xr3:uid="{0DE21D83-93B1-480C-BE9C-379DA0E532C7}" name="Missing" dataDxfId="63"/>
-    <tableColumn id="13" xr3:uid="{C4B407B9-B7FB-4DFC-A6B3-885C816BAF99}" name="Mean" dataDxfId="62"/>
-    <tableColumn id="14" xr3:uid="{9796FD8E-D568-43E1-AC6E-BFAE7C7B7017}" name="Median" dataDxfId="61"/>
-    <tableColumn id="15" xr3:uid="{A6A7BCED-DD2F-4B41-A84C-2F2674A38A53}" name="Mode" dataDxfId="60"/>
-    <tableColumn id="16" xr3:uid="{46607FA5-244C-49C2-997C-B64EB2E94FDE}" name="Standard Deviation" dataDxfId="59"/>
-    <tableColumn id="17" xr3:uid="{80BA1782-4C46-45CE-B3FB-40B70BA09AF9}" name="Variance" dataDxfId="58"/>
-    <tableColumn id="18" xr3:uid="{EC3C5A76-EF95-419C-87A8-D8885B542521}" name="Min" dataDxfId="57"/>
-    <tableColumn id="19" xr3:uid="{BFE545F8-810C-4F0A-A0B2-FF0AB9764A07}" name="5%" dataDxfId="56"/>
-    <tableColumn id="20" xr3:uid="{77D31A9B-57B1-4422-8EF9-6320F00E0DB9}" name="25%" dataDxfId="55"/>
-    <tableColumn id="21" xr3:uid="{7A350787-F0EA-4E65-B596-5D7253E75CD6}" name="50%" dataDxfId="54"/>
-    <tableColumn id="22" xr3:uid="{FB4C260E-A19F-4908-9DBF-DB4AC630982A}" name="75%" dataDxfId="53"/>
-    <tableColumn id="23" xr3:uid="{FBECC9F1-5BC8-4774-9475-EB2D6D28F1E2}" name="95%" dataDxfId="52"/>
-    <tableColumn id="24" xr3:uid="{839CD532-ED80-4544-A8C8-E9E036764A84}" name="Max" dataDxfId="51"/>
-    <tableColumn id="25" xr3:uid="{9DDA1FD6-82B1-4FBE-8BBD-B40C331930D2}" name="Range" dataDxfId="50"/>
-    <tableColumn id="26" xr3:uid="{902A027A-FD65-44D4-B3D0-5B3883ACFA39}" name="IQR" dataDxfId="49"/>
+    <tableColumn id="1" xr3:uid="{010A8E62-502A-4B19-B37A-BF59E03A068A}" name="Field" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{AD236665-EC7C-404F-8915-AD7CD5510D0F}" name="Definition" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{B78AB378-5727-433E-AB9C-BB970FC42B31}" name="Field Notes" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{EF15AE67-FE31-471E-840E-8104B878A3E8}" name="Data type" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{5006D683-9D12-4B97-9EF2-6D41AF6E0B35}" name="Distinct %" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{3AFB42F8-9976-44FF-9239-74914D5BE035}" name="Missing %" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{4BA41102-DB06-4180-9754-C88722FE82BD}" name="Memory Usage %" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{D22319BD-3A80-40F3-84FC-A6D1627B2F29}" name="Memory Usage" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{77FAEE19-B6C7-4056-8EF3-5EB877C820C4}" name="Distinct" dataDxfId="59"/>
+    <tableColumn id="10" xr3:uid="{54FF47BF-594E-417B-9028-64A4DFE4D389}" name="Count" dataDxfId="58"/>
+    <tableColumn id="11" xr3:uid="{54E587FE-36DC-4522-91DC-8B81B386217B}" name="Count %" dataDxfId="57"/>
+    <tableColumn id="12" xr3:uid="{0DE21D83-93B1-480C-BE9C-379DA0E532C7}" name="Missing" dataDxfId="56"/>
+    <tableColumn id="13" xr3:uid="{C4B407B9-B7FB-4DFC-A6B3-885C816BAF99}" name="Mean" dataDxfId="55"/>
+    <tableColumn id="14" xr3:uid="{9796FD8E-D568-43E1-AC6E-BFAE7C7B7017}" name="Median" dataDxfId="54"/>
+    <tableColumn id="15" xr3:uid="{A6A7BCED-DD2F-4B41-A84C-2F2674A38A53}" name="Mode" dataDxfId="53"/>
+    <tableColumn id="16" xr3:uid="{46607FA5-244C-49C2-997C-B64EB2E94FDE}" name="Standard Deviation" dataDxfId="52"/>
+    <tableColumn id="17" xr3:uid="{80BA1782-4C46-45CE-B3FB-40B70BA09AF9}" name="Variance" dataDxfId="51"/>
+    <tableColumn id="18" xr3:uid="{EC3C5A76-EF95-419C-87A8-D8885B542521}" name="Min" dataDxfId="50"/>
+    <tableColumn id="19" xr3:uid="{BFE545F8-810C-4F0A-A0B2-FF0AB9764A07}" name="5%" dataDxfId="49"/>
+    <tableColumn id="20" xr3:uid="{77D31A9B-57B1-4422-8EF9-6320F00E0DB9}" name="25%" dataDxfId="48"/>
+    <tableColumn id="21" xr3:uid="{7A350787-F0EA-4E65-B596-5D7253E75CD6}" name="50%" dataDxfId="47"/>
+    <tableColumn id="22" xr3:uid="{FB4C260E-A19F-4908-9DBF-DB4AC630982A}" name="75%" dataDxfId="46"/>
+    <tableColumn id="23" xr3:uid="{FBECC9F1-5BC8-4774-9475-EB2D6D28F1E2}" name="95%" dataDxfId="45"/>
+    <tableColumn id="24" xr3:uid="{839CD532-ED80-4544-A8C8-E9E036764A84}" name="Max" dataDxfId="44"/>
+    <tableColumn id="25" xr3:uid="{9DDA1FD6-82B1-4FBE-8BBD-B40C331930D2}" name="Range" dataDxfId="43"/>
+    <tableColumn id="26" xr3:uid="{902A027A-FD65-44D4-B3D0-5B3883ACFA39}" name="IQR" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D5F23AF2-1A5A-4EC2-A463-12BEF780B46A}" name="tbl_debug_section" displayName="tbl_debug_section" ref="C34:E41" totalsRowShown="0" headerRowDxfId="29" dataDxfId="27" headerRowBorderDxfId="28" tableBorderDxfId="26" totalsRowBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D5F23AF2-1A5A-4EC2-A463-12BEF780B46A}" name="tbl_debug_section" displayName="tbl_debug_section" ref="C34:E41" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19" totalsRowBorderDxfId="18">
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{FFACC0FF-000E-4785-9C1A-22F01E7C2644}" name="Production Section" dataDxfId="24" dataCellStyle="DarkHeader"/>
-    <tableColumn id="2" xr3:uid="{6A06C42D-D4AD-45CE-A81D-0918B410EAA9}" name="Production Time in Seconds" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{2643AF23-A2E5-4438-810D-7531CB2D2E4E}" name="% of Production Time" dataDxfId="22" dataCellStyle="Percent"/>
+    <tableColumn id="1" xr3:uid="{FFACC0FF-000E-4785-9C1A-22F01E7C2644}" name="Production Section" dataDxfId="17" dataCellStyle="DarkHeader"/>
+    <tableColumn id="2" xr3:uid="{6A06C42D-D4AD-45CE-A81D-0918B410EAA9}" name="Production Time in Seconds" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{2643AF23-A2E5-4438-810D-7531CB2D2E4E}" name="% of Production Time" dataDxfId="15" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E706681A-5322-4A3F-BB34-C5A4EED8E33F}" name="tbl_debug_environment" displayName="tbl_debug_environment" ref="C8:D23" totalsRowShown="0" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E706681A-5322-4A3F-BB34-C5A4EED8E33F}" name="tbl_debug_environment" displayName="tbl_debug_environment" ref="C8:D23" totalsRowShown="0" dataDxfId="13" headerRowBorderDxfId="14" tableBorderDxfId="12">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{9623C5AE-E7C2-4493-9B72-08667C9B2C60}" name="Environment Variable" dataDxfId="18" dataCellStyle="DarkHeader"/>
-    <tableColumn id="2" xr3:uid="{E5E357AA-48FB-47EA-928A-80845B0CD7C9}" name="Value" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{9623C5AE-E7C2-4493-9B72-08667C9B2C60}" name="Environment Variable" dataDxfId="11" dataCellStyle="DarkHeader"/>
+    <tableColumn id="2" xr3:uid="{E5E357AA-48FB-47EA-928A-80845B0CD7C9}" name="Value" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A6117933-3C15-4FC8-ADF4-0EC66304DEE1}" name="tbl_debug_config" displayName="tbl_debug_config" ref="F8:G10" totalsRowShown="0" headerRowBorderDxfId="16" tableBorderDxfId="15" totalsRowBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A6117933-3C15-4FC8-ADF4-0EC66304DEE1}" name="tbl_debug_config" displayName="tbl_debug_config" ref="F8:G10" totalsRowShown="0" headerRowBorderDxfId="9" tableBorderDxfId="8" totalsRowBorderDxfId="7">
   <autoFilter ref="F8:G10" xr:uid="{A6117933-3C15-4FC8-ADF4-0EC66304DEE1}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{EC70458D-5C3D-497C-AA06-AFCBD688FBDA}" name="Input Argument" dataDxfId="13" dataCellStyle="DarkHeader"/>
-    <tableColumn id="2" xr3:uid="{FCA8AE27-3D46-4152-9A03-0F3EFBA2366A}" name="Value" dataDxfId="12" dataCellStyle="DarkHeader"/>
+    <tableColumn id="1" xr3:uid="{EC70458D-5C3D-497C-AA06-AFCBD688FBDA}" name="Input Argument" dataDxfId="6" dataCellStyle="DarkHeader"/>
+    <tableColumn id="2" xr3:uid="{FCA8AE27-3D46-4152-9A03-0F3EFBA2366A}" name="Value" dataDxfId="5" dataCellStyle="DarkHeader"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6AF89CD0-DF40-4046-87D4-2BF660DDE636}" name="tbl_debug_errors" displayName="tbl_debug_errors" ref="I8:J10" totalsRowShown="0" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6AF89CD0-DF40-4046-87D4-2BF660DDE636}" name="tbl_debug_errors" displayName="tbl_debug_errors" ref="I8:J10" totalsRowShown="0" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
   <autoFilter ref="I8:J10" xr:uid="{6AF89CD0-DF40-4046-87D4-2BF660DDE636}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{27FA7240-202E-4FAB-AD4A-DC169AFD6F56}" name="Error Type" dataDxfId="8" dataCellStyle="DarkHeader"/>
-    <tableColumn id="2" xr3:uid="{C21354E4-3682-4AA0-B73A-2E689C89258C}" name="Detail" dataDxfId="7" dataCellStyle="DarkHeader"/>
+    <tableColumn id="1" xr3:uid="{27FA7240-202E-4FAB-AD4A-DC169AFD6F56}" name="Error Type" dataDxfId="1" dataCellStyle="DarkHeader"/>
+    <tableColumn id="2" xr3:uid="{C21354E4-3682-4AA0-B73A-2E689C89258C}" name="Detail" dataDxfId="0" dataCellStyle="DarkHeader"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3787,9 +3790,9 @@
     <tabColor rgb="FF000000"/>
   </sheetPr>
   <dimension ref="A1:W81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.6640625" defaultRowHeight="15" customHeight="1" outlineLevelRow="2" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="15.6640625" defaultRowHeight="15" customHeight="1" outlineLevelRow="2" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="0.83203125" customWidth="1"/>
+    <col min="1" max="1" width="0.77734375" customWidth="1"/>
     <col min="2" max="2" width="3" customWidth="1"/>
     <col min="3" max="3" width="2.6640625" customWidth="1"/>
     <col min="4" max="4" width="25.6640625" customWidth="1"/>
@@ -3797,7 +3800,7 @@
     <col min="8" max="8" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="20" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="17"/>
       <c r="B1" s="17"/>
       <c r="C1" s="18"/>
@@ -3824,8 +3827,8 @@
       <c r="V1" s="18"/>
       <c r="W1" s="18"/>
     </row>
-    <row r="2" spans="1:23" ht="10.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="1:23" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:23" ht="37.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>85</v>
       </c>
@@ -3834,8 +3837,8 @@
       </c>
       <c r="D3" s="26"/>
     </row>
-    <row r="4" spans="1:23" ht="10.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:23" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C5" s="64" t="s">
         <v>85</v>
       </c>
@@ -3843,46 +3846,46 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="10.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:23" ht="40" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:23" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:23" ht="40.049999999999997" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="E7" s="112" t="s">
         <v>59</v>
       </c>
       <c r="F7" s="113"/>
     </row>
-    <row r="8" spans="1:23" hidden="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="9" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:23" ht="14.4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D9" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E9" s="65"/>
     </row>
-    <row r="10" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D10" s="3" t="s">
         <v>55</v>
       </c>
       <c r="E10" s="33"/>
     </row>
-    <row r="11" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D11" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E11" s="33"/>
     </row>
-    <row r="12" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D12" s="3" t="s">
         <v>56</v>
       </c>
       <c r="E12" s="61"/>
     </row>
-    <row r="13" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:23" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D13" s="3" t="s">
         <v>57</v>
       </c>
       <c r="E13" s="62"/>
     </row>
-    <row r="14" spans="1:23" ht="10.25" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:23" ht="35" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:23" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:23" ht="34.950000000000003" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D15" s="25" t="s">
         <v>2</v>
       </c>
@@ -3896,8 +3899,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="10.25" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="17" spans="1:7" ht="35" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:23" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="1:7" ht="34.950000000000003" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D17" s="25" t="s">
         <v>3</v>
       </c>
@@ -3911,8 +3914,8 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="10.25" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="1:7" s="27" customFormat="1" ht="30" customHeight="1" collapsed="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="1:7" s="27" customFormat="1" ht="30" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A19"/>
       <c r="B19"/>
       <c r="C19" s="30"/>
@@ -3923,8 +3926,8 @@
       <c r="F19" s="31"/>
       <c r="G19" s="31"/>
     </row>
-    <row r="20" spans="1:7" ht="10.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="1:7" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" spans="1:7" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C21" s="64" t="s">
         <v>85</v>
       </c>
@@ -3932,8 +3935,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="10.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ht="10.199999999999999" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="23" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D23" s="23" t="s">
         <v>8</v>
       </c>
@@ -3941,7 +3944,7 @@
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
     </row>
-    <row r="24" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D24" s="3" t="s">
         <v>9</v>
       </c>
@@ -3949,7 +3952,7 @@
       <c r="F24" s="14"/>
       <c r="G24" s="14"/>
     </row>
-    <row r="25" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D25" s="22" t="s">
         <v>10</v>
       </c>
@@ -3957,7 +3960,7 @@
       <c r="F25" s="14"/>
       <c r="G25" s="14"/>
     </row>
-    <row r="26" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D26" s="22" t="s">
         <v>11</v>
       </c>
@@ -3965,7 +3968,7 @@
       <c r="F26" s="14"/>
       <c r="G26" s="14"/>
     </row>
-    <row r="27" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D27" s="22" t="s">
         <v>12</v>
       </c>
@@ -3973,7 +3976,7 @@
       <c r="F27" s="15"/>
       <c r="G27" s="15"/>
     </row>
-    <row r="28" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D28" s="22" t="s">
         <v>13</v>
       </c>
@@ -3981,7 +3984,7 @@
       <c r="F28" s="15"/>
       <c r="G28" s="15"/>
     </row>
-    <row r="29" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D29" s="23" t="s">
         <v>14</v>
       </c>
@@ -3989,7 +3992,7 @@
       <c r="F29" s="15"/>
       <c r="G29" s="15"/>
     </row>
-    <row r="30" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D30" s="3" t="s">
         <v>15</v>
       </c>
@@ -3997,10 +4000,10 @@
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
     </row>
-    <row r="31" spans="1:7" ht="10.25" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:7" ht="150" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="33" spans="3:7" ht="10.25" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="34" spans="3:7" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:7" ht="150" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3"/>
+    <row r="33" spans="3:7" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="3:7" ht="14.4" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="C34" s="64" t="s">
         <v>85</v>
       </c>
@@ -4008,8 +4011,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="3:7" ht="10.25" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="36" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:7" ht="10.199999999999999" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D36" s="3" t="s">
         <v>17</v>
       </c>
@@ -4017,7 +4020,7 @@
       <c r="F36" s="16"/>
       <c r="G36" s="16"/>
     </row>
-    <row r="37" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D37" s="22" t="s">
         <v>18</v>
       </c>
@@ -4025,7 +4028,7 @@
       <c r="F37" s="16"/>
       <c r="G37" s="16"/>
     </row>
-    <row r="38" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="38" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D38" s="22" t="s">
         <v>19</v>
       </c>
@@ -4033,7 +4036,7 @@
       <c r="F38" s="16"/>
       <c r="G38" s="16"/>
     </row>
-    <row r="39" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="39" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D39" s="3" t="s">
         <v>20</v>
       </c>
@@ -4041,7 +4044,7 @@
       <c r="F39" s="16"/>
       <c r="G39" s="16"/>
     </row>
-    <row r="40" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="40" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D40" s="24" t="s">
         <v>21</v>
       </c>
@@ -4049,10 +4052,10 @@
       <c r="F40" s="16"/>
       <c r="G40" s="16"/>
     </row>
-    <row r="41" spans="3:7" ht="10.25" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="3:7" ht="150" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="3:7" ht="10.25" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="3:7" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="3:7" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="3:7" ht="150" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="3:7" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="3:7" ht="14.4" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="C44" s="64" t="s">
         <v>85</v>
       </c>
@@ -4060,8 +4063,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="45" spans="3:7" ht="10" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="45" spans="3:7" ht="10.050000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D46" s="3" t="s">
         <v>23</v>
       </c>
@@ -4069,7 +4072,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="16"/>
     </row>
-    <row r="47" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="47" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D47" s="22">
         <v>0.05</v>
       </c>
@@ -4077,7 +4080,7 @@
       <c r="F47" s="16"/>
       <c r="G47" s="16"/>
     </row>
-    <row r="48" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="48" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D48" s="23">
         <v>0.25</v>
       </c>
@@ -4085,7 +4088,7 @@
       <c r="F48" s="16"/>
       <c r="G48" s="16"/>
     </row>
-    <row r="49" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="49" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D49" s="3">
         <v>0.5</v>
       </c>
@@ -4093,7 +4096,7 @@
       <c r="F49" s="16"/>
       <c r="G49" s="16"/>
     </row>
-    <row r="50" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D50" s="22">
         <v>0.75</v>
       </c>
@@ -4101,7 +4104,7 @@
       <c r="F50" s="16"/>
       <c r="G50" s="16"/>
     </row>
-    <row r="51" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="51" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D51" s="22">
         <v>0.95</v>
       </c>
@@ -4109,7 +4112,7 @@
       <c r="F51" s="16"/>
       <c r="G51" s="16"/>
     </row>
-    <row r="52" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="52" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D52" s="3" t="s">
         <v>24</v>
       </c>
@@ -4117,7 +4120,7 @@
       <c r="F52" s="16"/>
       <c r="G52" s="16"/>
     </row>
-    <row r="53" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="53" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D53" s="22" t="s">
         <v>25</v>
       </c>
@@ -4125,7 +4128,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="16"/>
     </row>
-    <row r="54" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D54" s="3" t="s">
         <v>26</v>
       </c>
@@ -4133,8 +4136,8 @@
       <c r="F54" s="16"/>
       <c r="G54" s="16"/>
     </row>
-    <row r="55" spans="3:7" ht="10.25" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="56" spans="3:7" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="3:7" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="3:7" ht="14.4" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="C56" s="64" t="s">
         <v>85</v>
       </c>
@@ -4142,8 +4145,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="57" spans="3:7" ht="10" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="58" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="57" spans="3:7" ht="10.050000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D58" s="3" t="s">
         <v>28</v>
       </c>
@@ -4157,7 +4160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="59" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D59" s="22" t="s">
         <v>29</v>
       </c>
@@ -4171,7 +4174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="60" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D60" s="22" t="s">
         <v>30</v>
       </c>
@@ -4185,7 +4188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="61" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D61" s="22" t="s">
         <v>31</v>
       </c>
@@ -4199,7 +4202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="62" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D62" s="3" t="s">
         <v>32</v>
       </c>
@@ -4213,7 +4216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="63" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D63" s="22" t="s">
         <v>33</v>
       </c>
@@ -4227,7 +4230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="64" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D64" s="22" t="s">
         <v>34</v>
       </c>
@@ -4241,7 +4244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="65" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D65" s="3" t="s">
         <v>35</v>
       </c>
@@ -4255,8 +4258,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="3:7" ht="10.25" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="67" spans="3:7" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="3:7" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3"/>
+    <row r="67" spans="3:7" ht="14.4" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="C67" s="64" t="s">
         <v>85</v>
       </c>
@@ -4264,8 +4267,8 @@
         <v>36</v>
       </c>
     </row>
-    <row r="68" spans="3:7" ht="10" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="69" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="68" spans="3:7" ht="10.050000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3"/>
+    <row r="69" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D69" s="3" t="str">
         <f>IF(COUNTIF(FieldList1, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(D58)," ","_") &amp;" = ")</f>
         <v/>
@@ -4275,7 +4278,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="70" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D70" s="21" t="str">
         <f>IF(COUNTIF(FieldList2, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(D59)," ","_")&amp;" = ")</f>
         <v/>
@@ -4285,7 +4288,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="71" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D71" s="21" t="str">
         <f>IF(COUNTIF(FieldList3, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(D60)," ","_")&amp;" = ")</f>
         <v/>
@@ -4295,7 +4298,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="72" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D72" s="21" t="str">
         <f>IF(COUNTIF(FieldList4, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(D61)," ","_")&amp;" = ")</f>
         <v/>
@@ -4305,7 +4308,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="73" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D73" s="21" t="str">
         <f>IF(COUNTIF(FieldList5, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(D62)," ","_")&amp;" = ")</f>
         <v/>
@@ -4315,7 +4318,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="74" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D74" s="21" t="str">
         <f>IF(COUNTIF(FieldList6, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(D63)," ","_")&amp;" = ")</f>
         <v/>
@@ -4325,7 +4328,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="75" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D75" s="20" t="str">
         <f>IF(COUNTIF(FieldList7, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(D64)," ","_")&amp;" = ")</f>
         <v/>
@@ -4335,7 +4338,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="76" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D76" s="3" t="str">
         <f>IF(COUNTIF(FieldList8, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(D65)," ","_")&amp;" = ")</f>
         <v/>
@@ -4345,7 +4348,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.2">
+    <row r="77" spans="3:7" ht="15" hidden="1" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="D77" s="19" t="str">
         <f>IF(COUNTIF(tbl_SourceData[Record List], "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(LightHeader)," ", "_") &amp;" = ")</f>
         <v/>
@@ -4355,8 +4358,8 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="3:7" ht="10.25" hidden="1" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2"/>
-    <row r="79" spans="3:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="3:7" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3"/>
+    <row r="79" spans="3:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D79" s="38" t="s">
         <v>37</v>
       </c>
@@ -4370,7 +4373,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="80" spans="3:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="3:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D80" s="57" t="b">
         <v>0</v>
       </c>
@@ -4378,7 +4381,7 @@
       <c r="F80" s="49"/>
       <c r="G80" s="49"/>
     </row>
-    <row r="81" spans="4:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="4:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D81" s="57" t="b">
         <v>0</v>
       </c>
@@ -4390,42 +4393,19 @@
   <mergeCells count="1">
     <mergeCell ref="E7:F7"/>
   </mergeCells>
-  <conditionalFormatting sqref="D79 D58:D65">
-    <cfRule type="duplicateValues" dxfId="6" priority="13"/>
+  <conditionalFormatting sqref="E23:G30 E36:G40 E46:G54">
+    <cfRule type="cellIs" dxfId="82" priority="19" operator="equal">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D80:D81">
-    <cfRule type="cellIs" dxfId="5" priority="18" operator="notEqual">
+    <cfRule type="cellIs" dxfId="81" priority="18" operator="notEqual">
       <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E7">
-    <cfRule type="cellIs" dxfId="4" priority="10" operator="notEqual">
-      <formula>"Dataset Description"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E12:E13">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.2"/>
-        <color theme="1" tint="-0.499984740745262"/>
-        <color rgb="FF7A0000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E15:G15">
-    <cfRule type="cellIs" dxfId="3" priority="11" operator="notEqual">
-      <formula>"Definition"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E17:G17">
-    <cfRule type="cellIs" dxfId="2" priority="12" operator="notEqual">
+    <cfRule type="cellIs" dxfId="80" priority="12" operator="notEqual">
       <formula>"Note"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23:G30 E36:G40 E46:G54">
-    <cfRule type="cellIs" dxfId="1" priority="19" operator="equal">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24:G26">
@@ -4438,9 +4418,32 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D79 D58:D65">
+    <cfRule type="duplicateValues" dxfId="79" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15:G15">
+    <cfRule type="cellIs" dxfId="78" priority="11" operator="notEqual">
+      <formula>"Definition"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="cellIs" dxfId="77" priority="10" operator="notEqual">
+      <formula>"Dataset Description"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E58:G65">
-    <cfRule type="cellIs" dxfId="0" priority="16" operator="notEqual">
+    <cfRule type="cellIs" dxfId="76" priority="16" operator="notEqual">
       <formula>FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12:E13">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.2"/>
+        <color theme="1" tint="-0.499984740745262"/>
+        <color rgb="FF7A0000"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4457,22 +4460,22 @@
     <tabColor rgb="FF000000"/>
   </sheetPr>
   <dimension ref="A1:AA12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="42.33203125" customWidth="1"/>
-    <col min="4" max="4" width="45.5" customWidth="1"/>
+    <col min="4" max="4" width="45.44140625" customWidth="1"/>
     <col min="5" max="5" width="17.6640625" customWidth="1"/>
-    <col min="6" max="7" width="15.83203125" customWidth="1"/>
+    <col min="6" max="7" width="15.77734375" customWidth="1"/>
     <col min="8" max="8" width="17.6640625" customWidth="1"/>
     <col min="9" max="9" width="15.6640625" customWidth="1"/>
-    <col min="10" max="16" width="13.5" customWidth="1"/>
+    <col min="10" max="16" width="13.44140625" customWidth="1"/>
     <col min="17" max="17" width="19" customWidth="1"/>
-    <col min="18" max="27" width="13.5" customWidth="1"/>
+    <col min="18" max="27" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="20" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="17"/>
       <c r="B1" s="18" t="s">
         <v>0</v>
@@ -4503,51 +4506,51 @@
       <c r="Z1" s="18"/>
       <c r="AA1" s="18"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="1:27" ht="36.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:27" ht="36.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="7" t="str">
         <f>'Field Analysis'!Name</f>
         <v>Name</v>
       </c>
       <c r="AA3" s="5"/>
     </row>
-    <row r="4" spans="1:27" ht="10.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="AA4" s="5"/>
     </row>
-    <row r="5" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="35" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="32"/>
       <c r="AA5" s="6"/>
     </row>
-    <row r="6" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="34" t="s">
         <v>55</v>
       </c>
       <c r="C6" s="33"/>
     </row>
-    <row r="7" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="34" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="33"/>
     </row>
-    <row r="8" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="34" t="s">
         <v>56</v>
       </c>
       <c r="C8" s="61"/>
     </row>
-    <row r="9" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="36" t="s">
         <v>57</v>
       </c>
       <c r="C9" s="62"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:27" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:27" ht="40.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27" ht="24" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:27" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="55" t="s">
         <v>41</v>
       </c>
@@ -4627,7 +4630,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="50"/>
       <c r="C12" s="63"/>
       <c r="D12" s="63"/>
@@ -4690,16 +4693,16 @@
     <tabColor rgb="FF000000"/>
   </sheetPr>
   <dimension ref="A1:Q10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="2.6640625" customWidth="1"/>
     <col min="3" max="5" width="12.6640625" customWidth="1"/>
     <col min="6" max="9" width="9.33203125" customWidth="1"/>
     <col min="10" max="10" width="10.6640625" customWidth="1"/>
-    <col min="11" max="16" width="15.5" customWidth="1"/>
+    <col min="11" max="16" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="20" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="17"/>
       <c r="B1" s="18" t="s">
         <v>0</v>
@@ -4720,21 +4723,21 @@
       <c r="P1" s="18"/>
       <c r="Q1" s="18"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" ht="14.4" x14ac:dyDescent="0.3">
       <c r="C2" s="9"/>
       <c r="D2" s="10"/>
     </row>
-    <row r="3" spans="1:17" ht="37" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" ht="36.6" x14ac:dyDescent="0.3">
       <c r="C3" s="7" t="str">
         <f>'Field Analysis'!Name</f>
         <v>Name</v>
       </c>
       <c r="P3" s="8"/>
     </row>
-    <row r="4" spans="1:17" ht="10.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D4" s="11"/>
     </row>
-    <row r="5" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="30"/>
       <c r="C5" s="30"/>
       <c r="D5" s="30"/>
@@ -4752,10 +4755,10 @@
       <c r="P5" s="30"/>
       <c r="Q5" s="30"/>
     </row>
-    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="12"/>
     </row>
-    <row r="9" spans="1:17" ht="36.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="36.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C9" s="28" t="s">
         <v>49</v>
       </c>
@@ -4766,7 +4769,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C10" s="29"/>
       <c r="D10" s="58"/>
       <c r="E10" s="59"/>
@@ -4803,17 +4806,17 @@
     <tabColor rgb="FF5D1955"/>
   </sheetPr>
   <dimension ref="B1:Y49"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelRow="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" outlineLevelRow="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.5" customWidth="1"/>
-    <col min="2" max="2" width="2.83203125" customWidth="1"/>
-    <col min="3" max="4" width="25.83203125" style="81" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" style="81" customWidth="1"/>
-    <col min="6" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="84" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.44140625" customWidth="1"/>
+    <col min="2" max="2" width="2.77734375" customWidth="1"/>
+    <col min="3" max="4" width="25.77734375" style="81" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" style="81" customWidth="1"/>
+    <col min="6" max="11" width="20.77734375" customWidth="1"/>
+    <col min="12" max="84" width="24.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.3">
       <c r="F1" s="81"/>
       <c r="G1" s="81"/>
       <c r="H1" s="81"/>
@@ -4821,7 +4824,7 @@
       <c r="J1" s="81"/>
       <c r="K1" s="81"/>
     </row>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
       <c r="F2" s="81"/>
       <c r="G2" s="81"/>
       <c r="H2" s="81"/>
@@ -4829,7 +4832,7 @@
       <c r="J2" s="81"/>
       <c r="K2" s="81"/>
     </row>
-    <row r="3" spans="2:12" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:12" ht="37.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="108" t="s">
         <v>85</v>
       </c>
@@ -4844,7 +4847,7 @@
       <c r="J3" s="81"/>
       <c r="K3" s="81"/>
     </row>
-    <row r="4" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="F4" s="81"/>
       <c r="G4" s="81"/>
       <c r="H4" s="81"/>
@@ -4852,7 +4855,7 @@
       <c r="J4" s="81"/>
       <c r="K4" s="81"/>
     </row>
-    <row r="5" spans="2:12" ht="10" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:12" ht="10.050000000000001" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
       <c r="C5" s="82"/>
       <c r="D5" s="82"/>
@@ -4863,7 +4866,7 @@
       <c r="J5" s="81"/>
       <c r="K5" s="81"/>
     </row>
-    <row r="6" spans="2:12" ht="44" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:12" ht="43.95" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C6" s="115" t="s">
         <v>62</v>
       </c>
@@ -4879,7 +4882,7 @@
       <c r="J6" s="81"/>
       <c r="K6" s="81"/>
     </row>
-    <row r="7" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="F7" s="81"/>
       <c r="G7" s="81"/>
       <c r="H7" s="81"/>
@@ -4888,7 +4891,7 @@
       <c r="K7" s="81"/>
       <c r="L7" s="71"/>
     </row>
-    <row r="8" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C8" s="89" t="s">
         <v>65</v>
       </c>
@@ -4911,7 +4914,7 @@
       <c r="K8" s="81"/>
       <c r="L8" s="71"/>
     </row>
-    <row r="9" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C9" s="83"/>
       <c r="D9" s="84"/>
       <c r="F9" s="94"/>
@@ -4922,7 +4925,7 @@
       <c r="K9" s="81"/>
       <c r="L9" s="72"/>
     </row>
-    <row r="10" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C10" s="83"/>
       <c r="D10" s="84"/>
       <c r="F10" s="83"/>
@@ -4932,74 +4935,74 @@
       <c r="J10" s="96"/>
       <c r="K10" s="81"/>
     </row>
-    <row r="11" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C11" s="83"/>
       <c r="D11" s="84"/>
     </row>
-    <row r="12" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C12" s="83"/>
       <c r="D12" s="84"/>
     </row>
-    <row r="13" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C13" s="83"/>
       <c r="D13" s="84"/>
     </row>
-    <row r="14" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C14" s="83"/>
       <c r="D14" s="84"/>
     </row>
-    <row r="15" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C15" s="83"/>
       <c r="D15" s="84"/>
     </row>
-    <row r="16" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C16" s="83"/>
       <c r="D16" s="84"/>
     </row>
-    <row r="17" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C17" s="83"/>
       <c r="D17" s="84"/>
     </row>
-    <row r="18" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C18" s="83"/>
       <c r="D18" s="84"/>
     </row>
-    <row r="19" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B19" s="73"/>
       <c r="C19" s="83"/>
       <c r="D19" s="84"/>
     </row>
-    <row r="20" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C20" s="83"/>
       <c r="D20" s="84"/>
     </row>
-    <row r="21" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C21" s="83"/>
       <c r="D21" s="84"/>
     </row>
-    <row r="22" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C22" s="83"/>
       <c r="D22" s="84"/>
       <c r="K22" s="81"/>
     </row>
-    <row r="23" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C23" s="99"/>
       <c r="D23" s="84"/>
       <c r="K23" s="81"/>
     </row>
-    <row r="24" spans="2:25" ht="30" hidden="1" customHeight="1" collapsed="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:25" ht="30" hidden="1" customHeight="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="B24" s="74"/>
       <c r="C24" s="85"/>
       <c r="E24" s="85"/>
       <c r="K24" s="81"/>
     </row>
-    <row r="25" spans="2:25" ht="10" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:25" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="74"/>
       <c r="C25" s="85"/>
       <c r="E25" s="85"/>
       <c r="K25" s="81"/>
     </row>
-    <row r="26" spans="2:25" ht="37" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:25" ht="37.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="26" t="s">
         <v>60</v>
       </c>
@@ -5009,7 +5012,7 @@
       </c>
       <c r="K26" s="81"/>
     </row>
-    <row r="27" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="76"/>
       <c r="F27" s="81"/>
       <c r="G27" s="81"/>
@@ -5019,7 +5022,7 @@
       <c r="K27" s="81"/>
       <c r="Y27" s="71"/>
     </row>
-    <row r="28" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C28" s="87" t="s">
         <v>67</v>
       </c>
@@ -5034,7 +5037,7 @@
       <c r="W28" s="76"/>
       <c r="Y28" s="71"/>
     </row>
-    <row r="29" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C29" s="87" t="s">
         <v>68</v>
       </c>
@@ -5049,7 +5052,7 @@
       <c r="X29" s="77"/>
       <c r="Y29" s="72"/>
     </row>
-    <row r="30" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C30" s="87" t="s">
         <v>69</v>
       </c>
@@ -5063,7 +5066,7 @@
       <c r="K30" s="81"/>
       <c r="X30" s="77"/>
     </row>
-    <row r="31" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C31" s="87" t="s">
         <v>70</v>
       </c>
@@ -5077,7 +5080,7 @@
       <c r="K31" s="88"/>
       <c r="X31" s="77"/>
     </row>
-    <row r="32" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C32" s="87" t="s">
         <v>71</v>
       </c>
@@ -5091,8 +5094,8 @@
       <c r="K32" s="88"/>
       <c r="X32" s="77"/>
     </row>
-    <row r="33" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" spans="2:5" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="2:5" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="75"/>
       <c r="C34" s="89" t="s">
         <v>72</v>
@@ -5104,83 +5107,83 @@
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C35" s="92" t="s">
         <v>75</v>
       </c>
       <c r="D35" s="102"/>
       <c r="E35" s="100"/>
     </row>
-    <row r="36" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C36" s="92" t="s">
         <v>76</v>
       </c>
       <c r="D36" s="102"/>
       <c r="E36" s="100"/>
     </row>
-    <row r="37" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C37" s="92" t="s">
         <v>77</v>
       </c>
       <c r="D37" s="102"/>
       <c r="E37" s="100"/>
     </row>
-    <row r="38" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C38" s="92" t="s">
         <v>78</v>
       </c>
       <c r="D38" s="102"/>
       <c r="E38" s="100"/>
     </row>
-    <row r="39" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C39" s="92" t="s">
         <v>79</v>
       </c>
       <c r="D39" s="102"/>
       <c r="E39" s="100"/>
     </row>
-    <row r="40" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C40" s="92" t="s">
         <v>80</v>
       </c>
       <c r="D40" s="102"/>
       <c r="E40" s="100"/>
     </row>
-    <row r="41" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C41" s="93" t="s">
         <v>81</v>
       </c>
       <c r="D41" s="103"/>
       <c r="E41" s="101"/>
     </row>
-    <row r="42" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C42" s="87"/>
       <c r="D42" s="104"/>
       <c r="E42" s="105"/>
     </row>
-    <row r="43" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C45"/>
       <c r="D45"/>
       <c r="E45"/>
     </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C46"/>
       <c r="D46"/>
       <c r="E46"/>
     </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C47"/>
       <c r="D47"/>
       <c r="E47"/>
     </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C48"/>
       <c r="D48"/>
       <c r="E48"/>
     </row>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="J26:J27"/>
@@ -5215,34 +5218,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725D1AF8-C53E-48B7-8625-1AC9E9368DD1}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="B2:P17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
     <col min="2" max="2" width="2.6640625" style="9" customWidth="1"/>
     <col min="3" max="3" width="78.6640625" style="10" customWidth="1"/>
-    <col min="4" max="4" width="31.83203125" customWidth="1"/>
+    <col min="4" max="4" width="31.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="43.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:16" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="39" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="2:16" ht="5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:16" ht="4.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3"/>
       <c r="C3" s="11"/>
       <c r="P3" s="8"/>
     </row>
-    <row r="4" spans="2:16" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4"/>
       <c r="C4" s="11"/>
       <c r="P4" s="40"/>
     </row>
-    <row r="5" spans="2:16" ht="5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:16" ht="4.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5"/>
       <c r="C5" s="11"/>
     </row>
-    <row r="6" spans="2:16" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:16" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="46"/>
       <c r="C6" s="47"/>
       <c r="D6" s="47"/>
@@ -5259,21 +5262,21 @@
       <c r="O6" s="47"/>
       <c r="P6" s="47"/>
     </row>
-    <row r="7" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7"/>
       <c r="C7"/>
     </row>
-    <row r="8" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="41"/>
     </row>
-    <row r="9" spans="2:16" ht="19.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:16" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9"/>
       <c r="C9" s="11"/>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C16"/>
     </row>
-    <row r="17" spans="2:2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B17" s="9"/>
     </row>
   </sheetData>
@@ -5286,7 +5289,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59DB964-5183-48E8-9EB0-23FD2468B797}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="B2:P20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="2.6640625" style="9" customWidth="1"/>
@@ -5294,29 +5297,29 @@
     <col min="4" max="4" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="51.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:16" ht="51.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="5"/>
       <c r="C2" s="39" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="2:16" ht="5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:16" ht="4.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5"/>
       <c r="C3" s="39"/>
       <c r="D3" s="42"/>
       <c r="P3" s="8"/>
     </row>
-    <row r="4" spans="2:16" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5"/>
       <c r="C4" s="39"/>
       <c r="D4" s="42"/>
       <c r="P4" s="40"/>
     </row>
-    <row r="5" spans="2:16" ht="5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:16" ht="4.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5"/>
       <c r="C5" s="11"/>
     </row>
-    <row r="6" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="46"/>
       <c r="C6" s="47"/>
       <c r="D6" s="47"/>
@@ -5333,38 +5336,38 @@
       <c r="O6" s="47"/>
       <c r="P6" s="47"/>
     </row>
-    <row r="7" spans="2:16" ht="10.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:16" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7"/>
       <c r="C7" s="11"/>
     </row>
-    <row r="8" spans="2:16" ht="10.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:16" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="8"/>
       <c r="D8" s="10"/>
     </row>
-    <row r="9" spans="2:16" ht="150" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:16" ht="150" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="43"/>
       <c r="C9" s="44"/>
     </row>
-    <row r="10" spans="2:16" ht="10.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:16" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="45"/>
     </row>
-    <row r="11" spans="2:16" collapsed="1" x14ac:dyDescent="0.2"/>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:16" collapsed="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C13"/>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C14"/>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C15"/>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="C16"/>
     </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C19"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C20"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed matplotlib headless implementation * Changed the plotting implementation to only use  a headless backend while producing plots.
</commit_message>
<xml_diff>
--- a/src/xleda/xleda_template.xlsx
+++ b/src/xleda/xleda_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B69C410F-6535-44B8-9CC6-BE281C12045F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD1132E3-4A4B-485D-B5ED-CA62EDE95C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Field Analysis" sheetId="25" r:id="rId1"/>

</xml_diff>

<commit_message>
Added http support for data/exporting, updated examples to have paths to data files on Github
</commit_message>
<xml_diff>
--- a/src/xleda/xleda_template.xlsx
+++ b/src/xleda/xleda_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\Python\.xleda\src\xleda\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{741A0408-1A40-410B-B64F-CE6CA3108EA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B780AAEB-3918-4B99-856C-722AC3079E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
   <sheets>
     <sheet name="SinglePlot" sheetId="30" state="hidden" r:id="rId1"/>
@@ -18,21 +18,21 @@
     <sheet name="Field Analysis" sheetId="25" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="Back">Overview!$D$57</definedName>
+    <definedName name="Back">Overview!$D$54</definedName>
     <definedName name="Compiled_Lists" localSheetId="2">'Field Analysis'!$C$71:$C$80</definedName>
     <definedName name="Composition" localSheetId="2">'Field Analysis'!$C$25:$C$35</definedName>
     <definedName name="CompositionTable" localSheetId="2">'Field Analysis'!$D$34</definedName>
     <definedName name="DarkHeader" localSheetId="2">'Field Analysis'!$D$81</definedName>
     <definedName name="Data_Description" localSheetId="2">'Field Analysis'!$C$9:$C$20</definedName>
-    <definedName name="Dataframes">Overview!$C$57:$C$60</definedName>
-    <definedName name="Debug" localSheetId="1">Overview!$D$9:$E$53</definedName>
+    <definedName name="Dataframes">Overview!$C$54:$C$57</definedName>
+    <definedName name="Debug" localSheetId="1">Overview!$D$9:$E$51</definedName>
     <definedName name="DebugToggle" localSheetId="1">Overview!$B$6</definedName>
     <definedName name="Definitions" localSheetId="2">'Field Analysis'!$D$17:$F$17</definedName>
     <definedName name="Description" localSheetId="2">'Field Analysis'!$D$9</definedName>
     <definedName name="Dimensions" localSheetId="2">'Field Analysis'!$D$11</definedName>
     <definedName name="Field_Analysis" localSheetId="2">'Field Analysis'!$D$22:$D$80</definedName>
     <definedName name="Field_Lists" localSheetId="2">'Field Analysis'!$C$60:$C$68</definedName>
-    <definedName name="Field_Overview">Overview!$E$64:$E$65</definedName>
+    <definedName name="Field_Overview">Overview!$E$61:$E$62</definedName>
     <definedName name="FieldList1" localSheetId="2">'Field Analysis'!$D$60:$F$60</definedName>
     <definedName name="FieldList2" localSheetId="2">'Field Analysis'!$D$61:$F$61</definedName>
     <definedName name="FieldList3" localSheetId="2">'Field Analysis'!$D$62:$F$62</definedName>
@@ -43,7 +43,7 @@
     <definedName name="FieldList8" localSheetId="2">'Field Analysis'!$D$67:$F$67</definedName>
     <definedName name="FieldLists" localSheetId="2">'Field Analysis'!$C$60:$F$67</definedName>
     <definedName name="FieldRange" localSheetId="2">'Field Analysis'!$D$81:$F$81</definedName>
-    <definedName name="Fields">Overview!$C$64:$C$65</definedName>
+    <definedName name="Fields">Overview!$C$61:$C$62</definedName>
     <definedName name="FormatRange" localSheetId="2">'Field Analysis'!$F:$F</definedName>
     <definedName name="Headers" localSheetId="2">'Field Analysis'!$D$21:$F$21</definedName>
     <definedName name="Headers_Start" localSheetId="2">'Field Analysis'!$D$21</definedName>
@@ -58,13 +58,13 @@
     <definedName name="SinglePlot" localSheetId="0">SinglePlot!$C$10</definedName>
     <definedName name="Summary_Stats" localSheetId="2">'Field Analysis'!$C$38:$C$45</definedName>
     <definedName name="Theme" localSheetId="2">'Field Analysis'!$B$21:$F$21</definedName>
-    <definedName name="Theme" localSheetId="1">Overview!$E$64:$AD$64</definedName>
+    <definedName name="Theme" localSheetId="1">Overview!$E$61:$AD$61</definedName>
     <definedName name="Theme" localSheetId="0">SinglePlot!$B$8:$P$8</definedName>
     <definedName name="Toggles" localSheetId="2">'Field Analysis'!$B$7,'Field Analysis'!$B$23,'Field Analysis'!$B$36,'Field Analysis'!$B$46,'Field Analysis'!$B$58,'Field Analysis'!$B$69</definedName>
     <definedName name="TopToggle" localSheetId="2">'Field Analysis'!$B$5</definedName>
     <definedName name="Warning" localSheetId="2">'Field Analysis'!$D$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -125,7 +125,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="106">
   <si>
     <t>Warning</t>
   </si>
@@ -304,18 +304,12 @@
     <t>% of Production Time</t>
   </si>
   <si>
-    <t>Creating Workbook</t>
-  </si>
-  <si>
     <t>Adding Plots</t>
   </si>
   <si>
     <t>Input Argument</t>
   </si>
   <si>
-    <t>Detail</t>
-  </si>
-  <si>
     <t>►</t>
   </si>
   <si>
@@ -430,22 +424,25 @@
     <t>Subsampled</t>
   </si>
   <si>
-    <t>Preparing Data</t>
-  </si>
-  <si>
     <t>Field Analysis</t>
   </si>
   <si>
     <t>Dataframe Description</t>
   </si>
   <si>
-    <t>Errors</t>
-  </si>
-  <si>
-    <t>Error</t>
-  </si>
-  <si>
-    <t>path</t>
+    <t>Initializing wb Components</t>
+  </si>
+  <si>
+    <t>Adding Data</t>
+  </si>
+  <si>
+    <t>file path</t>
+  </si>
+  <si>
+    <t>settings path</t>
+  </si>
+  <si>
+    <t>data argument</t>
   </si>
 </sst>
 </file>
@@ -788,7 +785,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1025,17 +1022,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color theme="1" tint="-0.499984740745262"/>
-      </right>
-      <top style="thin">
-        <color theme="1" tint="-0.499984740745262"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color theme="1" tint="-0.499984740745262"/>
       </left>
@@ -1077,7 +1063,7 @@
     </xf>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" textRotation="180"/>
@@ -1211,9 +1197,6 @@
     <xf numFmtId="3" fontId="10" fillId="8" borderId="16" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="8" borderId="21" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="164" fontId="18" fillId="2" borderId="20" xfId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1261,7 +1244,7 @@
     <xf numFmtId="3" fontId="10" fillId="8" borderId="12" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="8" borderId="22" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="8" borderId="21" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1"/>
@@ -1307,9 +1290,6 @@
     <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1389,7 +1369,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1407,9 +1387,6 @@
     </xf>
     <xf numFmtId="3" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="32" fillId="2" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1426,7 +1403,7 @@
     <cellStyle name="SubItem" xfId="4" xr:uid="{D21B07FD-5F6D-4154-8AB7-63D035214F3C}"/>
     <cellStyle name="SubSectionTItle" xfId="3" xr:uid="{8B04109E-AD21-4C71-8EF5-077A68DD2476}"/>
   </cellStyles>
-  <dxfs count="97">
+  <dxfs count="90">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3410,135 +3387,6 @@
           <color theme="1" tint="-0.249977111117893"/>
         </horizontal>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </left>
-        <right style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </right>
-        <top style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </top>
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="1" tint="-0.499984740745262"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1" tint="0.39997558519241921"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -4161,17 +4009,17 @@
   </dxfs>
   <tableStyles count="3" defaultTableStyle="DarkTable" defaultPivotStyle="DarkPivot">
     <tableStyle name="DarkPivot" table="0" count="3" xr9:uid="{F2CB4A64-8CC4-48DA-B721-DC29E793B33C}">
-      <tableStyleElement type="wholeTable" dxfId="96"/>
-      <tableStyleElement type="headerRow" dxfId="95"/>
-      <tableStyleElement type="totalRow" dxfId="94"/>
+      <tableStyleElement type="wholeTable" dxfId="89"/>
+      <tableStyleElement type="headerRow" dxfId="88"/>
+      <tableStyleElement type="totalRow" dxfId="87"/>
     </tableStyle>
     <tableStyle name="DarkTable" pivot="0" count="2" xr9:uid="{97C242D2-6F6D-4549-9428-17456D609B35}">
-      <tableStyleElement type="wholeTable" dxfId="93"/>
-      <tableStyleElement type="headerRow" dxfId="92"/>
+      <tableStyleElement type="wholeTable" dxfId="86"/>
+      <tableStyleElement type="headerRow" dxfId="85"/>
     </tableStyle>
     <tableStyle name="SlicerStyleDark" pivot="0" table="0" count="10" xr9:uid="{11F1E452-086F-4069-BF08-FF8656253E5D}">
-      <tableStyleElement type="wholeTable" dxfId="91"/>
-      <tableStyleElement type="headerRow" dxfId="90"/>
+      <tableStyleElement type="wholeTable" dxfId="84"/>
+      <tableStyleElement type="headerRow" dxfId="83"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -4505,48 +4353,38 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E2133564-163D-4CB0-A97C-9358270F5F9C}" name="tbl_debug_section" displayName="tbl_debug_section" ref="D11:F15" totalsRowShown="0" headerRowDxfId="82" dataDxfId="80" headerRowBorderDxfId="81" tableBorderDxfId="79" totalsRowBorderDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E2133564-163D-4CB0-A97C-9358270F5F9C}" name="tbl_debug_section" displayName="tbl_debug_section" ref="D11:F14" totalsRowShown="0" headerRowDxfId="75" dataDxfId="73" headerRowBorderDxfId="74" tableBorderDxfId="72" totalsRowBorderDxfId="71">
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{5EB43B6F-4FF7-4D4C-8202-BD94842B8017}" name="Production Section" dataDxfId="77" dataCellStyle="DarkHeader"/>
-    <tableColumn id="2" xr3:uid="{71F0A434-8F03-4CF9-987C-D6F88D936E0A}" name="Production Time in Seconds" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{507EC883-FE9F-434C-8323-6EBB4691FEEE}" name="% of Production Time" dataDxfId="75" dataCellStyle="Percent"/>
+    <tableColumn id="1" xr3:uid="{5EB43B6F-4FF7-4D4C-8202-BD94842B8017}" name="Production Section" dataDxfId="70" dataCellStyle="DarkHeader"/>
+    <tableColumn id="2" xr3:uid="{71F0A434-8F03-4CF9-987C-D6F88D936E0A}" name="Production Time in Seconds" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{507EC883-FE9F-434C-8323-6EBB4691FEEE}" name="% of Production Time" dataDxfId="68" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FABCC19D-29F4-4A1C-9C2C-61132A93E32D}" name="tbl_debug_environment" displayName="tbl_debug_environment" ref="D20:E35" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FABCC19D-29F4-4A1C-9C2C-61132A93E32D}" name="tbl_debug_environment" displayName="tbl_debug_environment" ref="D19:E33" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{6A891059-3C09-438F-9AB9-42F8BA5B3379}" name="Environment Variable" dataDxfId="70" dataCellStyle="DarkHeader"/>
-    <tableColumn id="2" xr3:uid="{D9E0C91D-D549-4194-8575-1343B51883A7}" name="Value" dataDxfId="69"/>
+    <tableColumn id="1" xr3:uid="{6A891059-3C09-438F-9AB9-42F8BA5B3379}" name="Environment Variable" dataDxfId="63" dataCellStyle="DarkHeader"/>
+    <tableColumn id="2" xr3:uid="{D9E0C91D-D549-4194-8575-1343B51883A7}" name="Value" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{88D10CD5-62A0-484D-A455-84E38CB47746}" name="tbl_debug_config" displayName="tbl_debug_config" ref="D40:E50" totalsRowShown="0" headerRowDxfId="68" headerRowBorderDxfId="67" tableBorderDxfId="66" totalsRowBorderDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{88D10CD5-62A0-484D-A455-84E38CB47746}" name="tbl_debug_config" displayName="tbl_debug_config" ref="D38:E50" totalsRowShown="0" headerRowDxfId="61" headerRowBorderDxfId="60" tableBorderDxfId="59" totalsRowBorderDxfId="58">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{BAFB02A5-6AA3-46EF-A3FA-1FC44F32BBF4}" name="Input Argument" dataDxfId="64" dataCellStyle="DarkHeader"/>
-    <tableColumn id="2" xr3:uid="{402A365F-6164-4790-9B23-3CC27E2F5642}" name="Value" dataDxfId="63" dataCellStyle="DarkHeader"/>
+    <tableColumn id="1" xr3:uid="{BAFB02A5-6AA3-46EF-A3FA-1FC44F32BBF4}" name="Input Argument" dataDxfId="57" dataCellStyle="DarkHeader"/>
+    <tableColumn id="2" xr3:uid="{402A365F-6164-4790-9B23-3CC27E2F5642}" name="Value" dataDxfId="56" dataCellStyle="DarkHeader"/>
   </tableColumns>
   <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{F61B5A24-D54F-42D3-BE0F-EC150E72D6E4}" name="tbl_debug_errors" displayName="tbl_debug_errors" ref="H11:I12" totalsRowShown="0" headerRowDxfId="62" dataDxfId="60" headerRowBorderDxfId="61" tableBorderDxfId="59" totalsRowBorderDxfId="58">
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{CA519729-E316-4F10-9FC9-4DAD4EBFD7D6}" name="Detail" dataDxfId="57" dataCellStyle="DarkHeader"/>
-    <tableColumn id="2" xr3:uid="{E2631007-AAAB-4565-904C-CFF05E0A66F2}" name="Error" dataDxfId="56" dataCellStyle="DarkHeader"/>
-  </tableColumns>
-  <tableStyleInfo name="DarkTable" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AFE650AA-A988-4967-9BF1-5CBBD5AE48A6}" name="tbl_FieldOverview" displayName="tbl_FieldOverview" ref="C64:AD65" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AFE650AA-A988-4967-9BF1-5CBBD5AE48A6}" name="tbl_FieldOverview" displayName="tbl_FieldOverview" ref="C61:AD62" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54">
   <tableColumns count="28">
     <tableColumn id="1" xr3:uid="{BFB84B7E-8B25-47B3-90FE-AC7BFBAF30EB}" name="_" dataDxfId="52" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{50D3F477-2874-418A-8431-FEC88B724332}" name="Dataframe" dataDxfId="51"/>
@@ -4581,8 +4419,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B62C177-35BB-4328-A5E9-CE2D42C175A6}" name="tbl_DfOverview" displayName="tbl_DfOverview" ref="C57:K58" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B62C177-35BB-4328-A5E9-CE2D42C175A6}" name="tbl_DfOverview" displayName="tbl_DfOverview" ref="C54:K55" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{95AE6ED1-2225-487F-9D3B-3E94D426571D}" name="_" dataDxfId="21" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{19718F20-2450-421A-9215-32A414225B3E}" name="Dataframe" dataDxfId="20" dataCellStyle="Hyperlink"/>
@@ -4598,7 +4436,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DB1D1E60-5E37-456A-AD85-0649D531840E}" name="tbl_SourceData" displayName="tbl_SourceData" ref="C81:F83" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4" headerRowCellStyle="DarkHeader" dataCellStyle="Normal">
   <autoFilter ref="C81:F83" xr:uid="{DB1D1E60-5E37-456A-AD85-0649D531840E}"/>
   <tableColumns count="4">
@@ -4952,43 +4790,43 @@
     <tabColor rgb="FF131313"/>
   </sheetPr>
   <dimension ref="B1:P19"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="8.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" style="7" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" style="7" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" ht="4.95" customHeight="1"/>
-    <row r="2" spans="2:16" ht="14.4" customHeight="1">
-      <c r="B2" s="86" t="s">
-        <v>94</v>
-      </c>
-      <c r="D2" s="86"/>
-    </row>
-    <row r="3" spans="2:16" ht="10.050000000000001" customHeight="1">
-      <c r="B3" s="78"/>
+    <row r="1" spans="2:16" ht="4.9000000000000004" customHeight="1"/>
+    <row r="2" spans="2:16" ht="14.45" customHeight="1">
+      <c r="B2" s="84" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="84"/>
+    </row>
+    <row r="3" spans="2:16" ht="10.15" customHeight="1">
+      <c r="B3" s="77"/>
     </row>
     <row r="4" spans="2:16" ht="30" customHeight="1">
-      <c r="B4" s="111" t="e" vm="1">
+      <c r="B4" s="109" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C4" s="54" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" spans="2:16" ht="4.95" customHeight="1">
+      <c r="C4" s="53" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" ht="4.9000000000000004" customHeight="1">
       <c r="B5" s="1"/>
       <c r="C5" s="8"/>
       <c r="P5" s="5"/>
     </row>
-    <row r="6" spans="2:16" ht="19.95" customHeight="1">
+    <row r="6" spans="2:16" ht="19.899999999999999" customHeight="1">
       <c r="B6"/>
       <c r="C6" s="8"/>
       <c r="P6" s="25"/>
     </row>
-    <row r="7" spans="2:16" ht="4.95" customHeight="1">
+    <row r="7" spans="2:16" ht="4.9000000000000004" customHeight="1">
       <c r="B7"/>
       <c r="C7" s="8"/>
     </row>
@@ -5016,7 +4854,7 @@
     <row r="10" spans="2:16" ht="15" customHeight="1">
       <c r="C10" s="26"/>
     </row>
-    <row r="11" spans="2:16" ht="19.2" customHeight="1">
+    <row r="11" spans="2:16" ht="19.149999999999999" customHeight="1">
       <c r="B11"/>
       <c r="C11" s="8"/>
     </row>
@@ -5041,55 +4879,59 @@
     <tabColor theme="4"/>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:AE65"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
+  <dimension ref="A1:AE62"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="8.33203125" customWidth="1"/>
-    <col min="3" max="3" width="10.44140625" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="6" width="27.21875" customWidth="1"/>
-    <col min="7" max="11" width="19.5546875" customWidth="1"/>
-    <col min="12" max="19" width="17.109375" customWidth="1"/>
-    <col min="20" max="20" width="20.21875" customWidth="1"/>
-    <col min="21" max="30" width="17.109375" customWidth="1"/>
+    <col min="5" max="6" width="27.28515625" customWidth="1"/>
+    <col min="7" max="11" width="19.5703125" customWidth="1"/>
+    <col min="12" max="19" width="17.140625" customWidth="1"/>
+    <col min="20" max="20" width="20.28515625" customWidth="1"/>
+    <col min="21" max="30" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="87" customFormat="1" ht="4.95" customHeight="1"/>
-    <row r="2" spans="1:28" ht="14.4" customHeight="1">
-      <c r="A2" s="72"/>
-    </row>
-    <row r="3" spans="1:28" s="87" customFormat="1" ht="10.050000000000001" customHeight="1">
-      <c r="A3" s="72"/>
+    <row r="1" spans="1:28" s="85" customFormat="1" ht="4.9000000000000004" customHeight="1">
+      <c r="H1"/>
+      <c r="I1"/>
+      <c r="J1"/>
+    </row>
+    <row r="2" spans="1:28" ht="14.45" customHeight="1">
+      <c r="A2" s="71"/>
+    </row>
+    <row r="3" spans="1:28" s="85" customFormat="1" ht="10.15" customHeight="1">
+      <c r="A3" s="71"/>
+      <c r="H3"/>
+      <c r="I3"/>
+      <c r="J3"/>
     </row>
     <row r="4" spans="1:28" ht="30" customHeight="1">
-      <c r="B4" s="112" t="e" vm="1">
+      <c r="B4" s="110" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C4" s="54" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="75"/>
+      <c r="C4" s="53" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="74"/>
       <c r="AB4" s="4"/>
     </row>
-    <row r="5" spans="1:28" ht="10.050000000000001" customHeight="1">
-      <c r="C5" s="54"/>
+    <row r="5" spans="1:28" ht="10.15" customHeight="1">
+      <c r="C5" s="53"/>
       <c r="AB5" s="4"/>
     </row>
     <row r="6" spans="1:28" ht="15" customHeight="1">
-      <c r="B6" s="84" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="86" t="s">
-        <v>97</v>
-      </c>
-      <c r="D6" s="52"/>
+      <c r="B6" s="83" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="84" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="51"/>
       <c r="E6" s="43"/>
-      <c r="F6" s="53"/>
+      <c r="F6" s="52"/>
       <c r="G6" s="43"/>
-      <c r="H6" s="120"/>
-      <c r="I6" s="120"/>
-      <c r="J6" s="43"/>
       <c r="K6" s="43"/>
     </row>
     <row r="7" spans="1:28" ht="15" hidden="1" customHeight="1">
@@ -5098,9 +4940,6 @@
       <c r="E7" s="43"/>
       <c r="F7" s="43"/>
       <c r="G7" s="43"/>
-      <c r="H7" s="120"/>
-      <c r="I7" s="120"/>
-      <c r="J7" s="43"/>
       <c r="K7" s="43"/>
     </row>
     <row r="8" spans="1:28" ht="15" customHeight="1">
@@ -5108,141 +4947,122 @@
       <c r="D8" s="43"/>
       <c r="E8" s="43"/>
       <c r="F8" s="43"/>
-      <c r="G8" s="113"/>
-      <c r="H8" s="85"/>
-      <c r="I8" s="85"/>
-      <c r="J8" s="43"/>
+      <c r="G8" s="111"/>
       <c r="K8" s="43"/>
     </row>
     <row r="9" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="B9" s="1"/>
-      <c r="C9" s="121" t="s">
-        <v>99</v>
-      </c>
-      <c r="D9" s="121"/>
+      <c r="C9" s="118" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" s="118"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
-      <c r="H9" s="121" t="s">
-        <v>104</v>
-      </c>
-      <c r="I9" s="121"/>
-      <c r="J9" s="43"/>
       <c r="K9" s="43"/>
     </row>
-    <row r="10" spans="1:28" ht="4.95" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="10" spans="1:28" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
       <c r="C10" s="43"/>
       <c r="D10" s="43"/>
       <c r="E10" s="43"/>
     </row>
     <row r="11" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
       <c r="B11" s="41"/>
-      <c r="D11" s="115" t="s">
+      <c r="D11" s="113" t="s">
         <v>56</v>
       </c>
-      <c r="E11" s="117" t="s">
+      <c r="E11" s="115" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="116" t="s">
+      <c r="F11" s="114" t="s">
         <v>58</v>
       </c>
-      <c r="H11" s="115" t="s">
+    </row>
+    <row r="12" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D12" s="116" t="s">
+        <v>101</v>
+      </c>
+      <c r="E12" s="50"/>
+      <c r="F12" s="49"/>
+    </row>
+    <row r="13" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D13" s="116" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" s="50"/>
+      <c r="F13" s="49"/>
+    </row>
+    <row r="14" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D14" s="116" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="50"/>
+      <c r="F14" s="49"/>
+    </row>
+    <row r="15" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="43"/>
+    </row>
+    <row r="16" spans="1:28" ht="10.15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="L16" s="38"/>
+    </row>
+    <row r="17" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C17" s="118" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="118"/>
+      <c r="E17" s="80"/>
+      <c r="L17" s="38"/>
+    </row>
+    <row r="18" spans="2:12" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+    </row>
+    <row r="19" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D19" s="113" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="114" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D20" s="44" t="s">
         <v>62</v>
       </c>
-      <c r="I11" s="116" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D12" s="118" t="s">
-        <v>101</v>
-      </c>
-      <c r="E12" s="51"/>
-      <c r="F12" s="50"/>
-      <c r="H12" s="49"/>
-      <c r="I12" s="67"/>
-    </row>
-    <row r="13" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D13" s="118" t="s">
-        <v>59</v>
-      </c>
-      <c r="E13" s="51"/>
-      <c r="F13" s="50"/>
-    </row>
-    <row r="14" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D14" s="118" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="51"/>
-      <c r="F14" s="50"/>
-    </row>
-    <row r="15" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D15" s="118" t="s">
-        <v>60</v>
-      </c>
-      <c r="E15" s="51"/>
-      <c r="F15" s="50"/>
-    </row>
-    <row r="16" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C16" s="43"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
-    </row>
-    <row r="17" spans="2:12" ht="10.050000000000001" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="H17" s="82"/>
-      <c r="I17" s="83"/>
-      <c r="L17" s="38"/>
-    </row>
-    <row r="18" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C18" s="121" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="121"/>
-      <c r="E18" s="81"/>
-      <c r="L18" s="38"/>
-    </row>
-    <row r="19" spans="2:12" ht="4.95" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D19" s="43"/>
-      <c r="E19" s="43"/>
-    </row>
-    <row r="20" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D20" s="115" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="116" t="s">
-        <v>55</v>
-      </c>
+      <c r="E20" s="56"/>
     </row>
     <row r="21" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D21" s="44" t="s">
-        <v>64</v>
-      </c>
-      <c r="E21" s="57"/>
+        <v>63</v>
+      </c>
+      <c r="E21" s="56"/>
     </row>
     <row r="22" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D22" s="44" t="s">
-        <v>65</v>
-      </c>
-      <c r="E22" s="57"/>
+        <v>64</v>
+      </c>
+      <c r="E22" s="56"/>
     </row>
     <row r="23" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D23" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="E23" s="57"/>
+      <c r="E23" s="56"/>
     </row>
     <row r="24" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D24" s="44" t="s">
         <v>67</v>
       </c>
-      <c r="E24" s="57"/>
+      <c r="E24" s="56"/>
     </row>
     <row r="25" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D25" s="44" t="s">
         <v>68</v>
       </c>
-      <c r="E25" s="57"/>
+      <c r="E25" s="56"/>
     </row>
     <row r="26" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D26" s="44" t="s">
@@ -5254,77 +5074,88 @@
       <c r="D27" s="44" t="s">
         <v>70</v>
       </c>
-      <c r="E27" s="58"/>
+      <c r="E27" s="56"/>
     </row>
     <row r="28" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B28" s="39"/>
       <c r="D28" s="44" t="s">
         <v>71</v>
       </c>
-      <c r="E28" s="57"/>
+      <c r="E28" s="56"/>
     </row>
     <row r="29" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B29" s="39"/>
       <c r="D29" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="E29" s="57"/>
+      <c r="E29" s="56"/>
     </row>
     <row r="30" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D30" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="E30" s="57"/>
+      <c r="E30" s="56"/>
     </row>
     <row r="31" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D31" s="44" t="s">
         <v>74</v>
       </c>
-      <c r="E31" s="57"/>
+      <c r="E31" s="56"/>
+      <c r="I31" s="81"/>
+      <c r="J31" s="82"/>
+      <c r="K31" s="43"/>
     </row>
     <row r="32" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D32" s="44" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="57"/>
-      <c r="I32" s="82"/>
-      <c r="J32" s="83"/>
+      <c r="E32" s="56"/>
       <c r="K32" s="43"/>
     </row>
     <row r="33" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B33" s="40"/>
+      <c r="C33" s="45"/>
       <c r="D33" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="57"/>
+      <c r="E33" s="56"/>
       <c r="K33" s="43"/>
     </row>
     <row r="34" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="B34" s="40"/>
       <c r="C34" s="45"/>
-      <c r="D34" s="44" t="s">
-        <v>77</v>
-      </c>
-      <c r="E34" s="57"/>
+      <c r="D34" s="81"/>
+      <c r="E34" s="56"/>
       <c r="K34" s="43"/>
     </row>
     <row r="35" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B35" s="40"/>
-      <c r="C35" s="45"/>
-      <c r="D35" s="49" t="s">
-        <v>78</v>
-      </c>
-      <c r="E35" s="57"/>
+      <c r="D35" s="47"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="43"/>
       <c r="K35" s="43"/>
-    </row>
-    <row r="36" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B36" s="40"/>
-      <c r="C36" s="45"/>
-      <c r="D36" s="82"/>
-      <c r="E36" s="57"/>
+      <c r="W35" s="42"/>
+      <c r="Y35" s="38"/>
+    </row>
+    <row r="36" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C36" s="118" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" s="118"/>
+      <c r="F36" s="43"/>
+      <c r="G36" s="43"/>
+      <c r="H36" s="43"/>
+      <c r="I36" s="43"/>
+      <c r="J36" s="43"/>
       <c r="K36" s="43"/>
-    </row>
-    <row r="37" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D37" s="47"/>
-      <c r="E37" s="46"/>
+      <c r="W36" s="42"/>
+      <c r="Y36" s="38"/>
+    </row>
+    <row r="37" spans="2:25" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D37" s="43"/>
+      <c r="E37" s="43"/>
       <c r="F37" s="43"/>
       <c r="G37" s="43"/>
       <c r="H37" s="43"/>
@@ -5335,10 +5166,12 @@
       <c r="Y37" s="38"/>
     </row>
     <row r="38" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C38" s="121" t="s">
-        <v>53</v>
-      </c>
-      <c r="D38" s="121"/>
+      <c r="D38" s="113" t="s">
+        <v>60</v>
+      </c>
+      <c r="E38" s="114" t="s">
+        <v>55</v>
+      </c>
       <c r="F38" s="43"/>
       <c r="G38" s="43"/>
       <c r="H38" s="43"/>
@@ -5348,9 +5181,11 @@
       <c r="W38" s="42"/>
       <c r="Y38" s="38"/>
     </row>
-    <row r="39" spans="2:25" ht="4.95" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
+    <row r="39" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D39" s="48" t="s">
+        <v>103</v>
+      </c>
+      <c r="E39" s="54"/>
       <c r="F39" s="43"/>
       <c r="G39" s="43"/>
       <c r="H39" s="43"/>
@@ -5360,13 +5195,11 @@
       <c r="W39" s="42"/>
       <c r="Y39" s="38"/>
     </row>
-    <row r="40" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D40" s="115" t="s">
-        <v>61</v>
-      </c>
-      <c r="E40" s="116" t="s">
-        <v>55</v>
-      </c>
+    <row r="40" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D40" s="44" t="s">
+        <v>104</v>
+      </c>
+      <c r="E40" s="55"/>
       <c r="F40" s="43"/>
       <c r="G40" s="43"/>
       <c r="H40" s="43"/>
@@ -5377,8 +5210,8 @@
       <c r="Y40" s="38"/>
     </row>
     <row r="41" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D41" s="48" t="s">
-        <v>106</v>
+      <c r="D41" s="64" t="s">
+        <v>105</v>
       </c>
       <c r="E41" s="55"/>
       <c r="F41" s="43"/>
@@ -5391,10 +5224,10 @@
       <c r="Y41" s="38"/>
     </row>
     <row r="42" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D42" s="44" t="s">
-        <v>79</v>
-      </c>
-      <c r="E42" s="56"/>
+      <c r="D42" s="64" t="s">
+        <v>77</v>
+      </c>
+      <c r="E42" s="55"/>
       <c r="F42" s="43"/>
       <c r="G42" s="43"/>
       <c r="H42" s="43"/>
@@ -5405,10 +5238,10 @@
       <c r="Y42" s="38"/>
     </row>
     <row r="43" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D43" s="65" t="s">
-        <v>80</v>
-      </c>
-      <c r="E43" s="56"/>
+      <c r="D43" s="64" t="s">
+        <v>78</v>
+      </c>
+      <c r="E43" s="55"/>
       <c r="F43" s="43"/>
       <c r="G43" s="43"/>
       <c r="H43" s="43"/>
@@ -5419,10 +5252,10 @@
       <c r="Y43" s="38"/>
     </row>
     <row r="44" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D44" s="65" t="s">
-        <v>81</v>
-      </c>
-      <c r="E44" s="56"/>
+      <c r="D44" s="64" t="s">
+        <v>79</v>
+      </c>
+      <c r="E44" s="55"/>
       <c r="F44" s="43"/>
       <c r="G44" s="43"/>
       <c r="H44" s="43"/>
@@ -5433,10 +5266,10 @@
       <c r="Y44" s="38"/>
     </row>
     <row r="45" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D45" s="65" t="s">
-        <v>82</v>
-      </c>
-      <c r="E45" s="56"/>
+      <c r="D45" s="64" t="s">
+        <v>80</v>
+      </c>
+      <c r="E45" s="55"/>
       <c r="F45" s="43"/>
       <c r="G45" s="43"/>
       <c r="H45" s="43"/>
@@ -5447,10 +5280,10 @@
       <c r="Y45" s="38"/>
     </row>
     <row r="46" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D46" s="65" t="s">
-        <v>83</v>
-      </c>
-      <c r="E46" s="56"/>
+      <c r="D46" s="64" t="s">
+        <v>81</v>
+      </c>
+      <c r="E46" s="55"/>
       <c r="F46" s="43"/>
       <c r="G46" s="43"/>
       <c r="H46" s="43"/>
@@ -5461,10 +5294,10 @@
       <c r="Y46" s="38"/>
     </row>
     <row r="47" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D47" s="65" t="s">
-        <v>84</v>
-      </c>
-      <c r="E47" s="56"/>
+      <c r="D47" s="64" t="s">
+        <v>82</v>
+      </c>
+      <c r="E47" s="55"/>
       <c r="F47" s="43"/>
       <c r="G47" s="43"/>
       <c r="H47" s="43"/>
@@ -5476,9 +5309,9 @@
     </row>
     <row r="48" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D48" s="65" t="s">
-        <v>85</v>
-      </c>
-      <c r="E48" s="56"/>
+        <v>83</v>
+      </c>
+      <c r="E48" s="66"/>
       <c r="F48" s="43"/>
       <c r="G48" s="43"/>
       <c r="H48" s="43"/>
@@ -5489,10 +5322,10 @@
       <c r="Y48" s="38"/>
     </row>
     <row r="49" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D49" s="65" t="s">
-        <v>86</v>
-      </c>
-      <c r="E49" s="56"/>
+      <c r="D49" s="64" t="s">
+        <v>84</v>
+      </c>
+      <c r="E49" s="55"/>
       <c r="F49" s="43"/>
       <c r="G49" s="43"/>
       <c r="H49" s="43"/>
@@ -5503,10 +5336,10 @@
       <c r="Y49" s="38"/>
     </row>
     <row r="50" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D50" s="66" t="s">
-        <v>67</v>
-      </c>
-      <c r="E50" s="67"/>
+      <c r="D50" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="E50" s="66"/>
       <c r="F50" s="43"/>
       <c r="G50" s="43"/>
       <c r="H50" s="43"/>
@@ -5528,239 +5361,200 @@
       <c r="W51" s="42"/>
       <c r="Y51" s="38"/>
     </row>
-    <row r="52" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D52" s="47"/>
-      <c r="E52" s="46"/>
-      <c r="F52" s="43"/>
-      <c r="G52" s="43"/>
-      <c r="H52" s="43"/>
-      <c r="I52" s="43"/>
-      <c r="J52" s="43"/>
-      <c r="K52" s="43"/>
-      <c r="W52" s="42"/>
-      <c r="Y52" s="38"/>
-    </row>
-    <row r="53" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D53" s="47"/>
-      <c r="E53" s="46"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="43"/>
-      <c r="I53" s="43"/>
-      <c r="J53" s="43"/>
-      <c r="K53" s="43"/>
-      <c r="W53" s="42"/>
-      <c r="Y53" s="38"/>
-    </row>
-    <row r="54" spans="1:31" s="87" customFormat="1" ht="15" customHeight="1" collapsed="1">
-      <c r="D54" s="47"/>
-      <c r="E54" s="46"/>
-      <c r="F54" s="43"/>
-      <c r="G54" s="43"/>
-      <c r="H54" s="43"/>
-      <c r="I54" s="43"/>
-      <c r="J54" s="43"/>
-      <c r="K54" s="43"/>
-      <c r="W54" s="42"/>
-      <c r="Y54" s="38"/>
+    <row r="52" spans="1:31" ht="15" customHeight="1" collapsed="1">
+      <c r="A52" s="6"/>
+      <c r="B52" s="68" t="s">
+        <v>61</v>
+      </c>
+      <c r="C52" s="112" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB52" s="4"/>
+    </row>
+    <row r="53" spans="1:31" ht="15" customHeight="1">
+      <c r="C53" s="53"/>
+      <c r="AB53" s="4"/>
+    </row>
+    <row r="54" spans="1:31" ht="30" customHeight="1">
+      <c r="C54" s="88" t="s">
+        <v>91</v>
+      </c>
+      <c r="D54" s="89" t="s">
+        <v>86</v>
+      </c>
+      <c r="E54" s="90" t="s">
+        <v>100</v>
+      </c>
+      <c r="F54" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="G54" s="91" t="s">
+        <v>6</v>
+      </c>
+      <c r="H54" s="91" t="s">
+        <v>48</v>
+      </c>
+      <c r="I54" s="91" t="s">
+        <v>90</v>
+      </c>
+      <c r="J54" s="91" t="s">
+        <v>10</v>
+      </c>
+      <c r="K54" s="87" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE54" s="4"/>
     </row>
     <row r="55" spans="1:31" ht="15" customHeight="1">
-      <c r="A55" s="6"/>
-      <c r="B55" s="69" t="s">
-        <v>63</v>
-      </c>
-      <c r="C55" s="114" t="s">
-        <v>89</v>
-      </c>
-      <c r="AB55" s="4"/>
-    </row>
-    <row r="56" spans="1:31" ht="15" customHeight="1">
-      <c r="C56" s="54"/>
-      <c r="AB56" s="4"/>
-    </row>
-    <row r="57" spans="1:31" ht="30" customHeight="1">
-      <c r="C57" s="90" t="s">
-        <v>93</v>
-      </c>
-      <c r="D57" s="91" t="s">
+      <c r="C55" s="94"/>
+      <c r="D55" s="103"/>
+      <c r="E55" s="104"/>
+      <c r="F55" s="117"/>
+      <c r="G55" s="105"/>
+      <c r="H55" s="106"/>
+      <c r="I55" s="107"/>
+      <c r="J55" s="99"/>
+      <c r="K55" s="108"/>
+      <c r="AE55" s="4"/>
+    </row>
+    <row r="57" spans="1:31" ht="15" customHeight="1">
+      <c r="AB57" s="4"/>
+    </row>
+    <row r="58" spans="1:31" ht="15" customHeight="1">
+      <c r="B58" s="68" t="s">
+        <v>61</v>
+      </c>
+      <c r="C58" s="112" t="s">
         <v>88</v>
       </c>
-      <c r="E57" s="92" t="s">
-        <v>103</v>
-      </c>
-      <c r="F57" s="89" t="s">
+      <c r="D58" s="85"/>
+      <c r="AB58" s="4"/>
+    </row>
+    <row r="59" spans="1:31" ht="10.15" customHeight="1"/>
+    <row r="60" spans="1:31" ht="10.15" customHeight="1"/>
+    <row r="61" spans="1:31" ht="30" customHeight="1">
+      <c r="C61" s="88" t="s">
         <v>91</v>
       </c>
-      <c r="G57" s="93" t="s">
-        <v>6</v>
-      </c>
-      <c r="H57" s="93" t="s">
-        <v>48</v>
-      </c>
-      <c r="I57" s="93" t="s">
-        <v>92</v>
-      </c>
-      <c r="J57" s="93" t="s">
+      <c r="D61" s="92" t="s">
+        <v>86</v>
+      </c>
+      <c r="E61" s="92" t="s">
+        <v>39</v>
+      </c>
+      <c r="F61" s="92" t="s">
+        <v>40</v>
+      </c>
+      <c r="G61" s="92" t="s">
+        <v>1</v>
+      </c>
+      <c r="H61" s="87" t="s">
+        <v>8</v>
+      </c>
+      <c r="I61" s="87" t="s">
+        <v>9</v>
+      </c>
+      <c r="J61" s="87" t="s">
         <v>10</v>
       </c>
-      <c r="K57" s="89" t="s">
-        <v>100</v>
-      </c>
-      <c r="AE57" s="4"/>
-    </row>
-    <row r="58" spans="1:31" ht="15" customHeight="1">
-      <c r="C58" s="96"/>
-      <c r="D58" s="105"/>
-      <c r="E58" s="106"/>
-      <c r="F58" s="119"/>
-      <c r="G58" s="107"/>
-      <c r="H58" s="108"/>
-      <c r="I58" s="109"/>
-      <c r="J58" s="101"/>
-      <c r="K58" s="110"/>
-      <c r="AE58" s="4"/>
-    </row>
-    <row r="60" spans="1:31" ht="15" customHeight="1">
-      <c r="AB60" s="4"/>
-    </row>
-    <row r="61" spans="1:31" ht="15" customHeight="1">
-      <c r="B61" s="69" t="s">
-        <v>63</v>
-      </c>
-      <c r="C61" s="114" t="s">
-        <v>90</v>
-      </c>
-      <c r="D61" s="87"/>
-      <c r="AB61" s="4"/>
-    </row>
-    <row r="62" spans="1:31" ht="10.050000000000001" customHeight="1"/>
-    <row r="63" spans="1:31" ht="10.050000000000001" customHeight="1"/>
-    <row r="64" spans="1:31" ht="30" customHeight="1">
-      <c r="C64" s="90" t="s">
-        <v>93</v>
-      </c>
-      <c r="D64" s="94" t="s">
-        <v>88</v>
-      </c>
-      <c r="E64" s="94" t="s">
-        <v>39</v>
-      </c>
-      <c r="F64" s="94" t="s">
-        <v>40</v>
-      </c>
-      <c r="G64" s="94" t="s">
-        <v>1</v>
-      </c>
-      <c r="H64" s="89" t="s">
-        <v>8</v>
-      </c>
-      <c r="I64" s="89" t="s">
-        <v>9</v>
-      </c>
-      <c r="J64" s="89" t="s">
-        <v>10</v>
-      </c>
-      <c r="K64" s="89" t="s">
+      <c r="K61" s="87" t="s">
         <v>11</v>
       </c>
-      <c r="L64" s="89" t="s">
+      <c r="L61" s="87" t="s">
         <v>12</v>
       </c>
-      <c r="M64" s="89" t="s">
+      <c r="M61" s="87" t="s">
         <v>13</v>
       </c>
-      <c r="N64" s="89" t="s">
+      <c r="N61" s="87" t="s">
         <v>14</v>
       </c>
-      <c r="O64" s="89" t="s">
+      <c r="O61" s="87" t="s">
         <v>41</v>
       </c>
-      <c r="P64" s="89" t="s">
+      <c r="P61" s="87" t="s">
         <v>15</v>
       </c>
-      <c r="Q64" s="89" t="s">
+      <c r="Q61" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="R64" s="89" t="s">
+      <c r="R61" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="S64" s="89" t="s">
+      <c r="S61" s="87" t="s">
         <v>19</v>
       </c>
-      <c r="T64" s="89" t="s">
+      <c r="T61" s="87" t="s">
         <v>20</v>
       </c>
-      <c r="U64" s="89" t="s">
+      <c r="U61" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="V64" s="89" t="s">
+      <c r="V61" s="87" t="s">
         <v>23</v>
       </c>
-      <c r="W64" s="95" t="s">
+      <c r="W61" s="93" t="s">
         <v>42</v>
       </c>
-      <c r="X64" s="95" t="s">
+      <c r="X61" s="93" t="s">
         <v>43</v>
       </c>
-      <c r="Y64" s="95" t="s">
+      <c r="Y61" s="93" t="s">
         <v>44</v>
       </c>
-      <c r="Z64" s="95" t="s">
+      <c r="Z61" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="AA64" s="95" t="s">
+      <c r="AA61" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="AB64" s="89" t="s">
+      <c r="AB61" s="87" t="s">
         <v>24</v>
       </c>
-      <c r="AC64" s="89" t="s">
+      <c r="AC61" s="87" t="s">
         <v>25</v>
       </c>
-      <c r="AD64" s="89" t="s">
+      <c r="AD61" s="87" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="65" spans="3:30" ht="15" customHeight="1">
-      <c r="C65" s="96"/>
-      <c r="D65" s="97"/>
-      <c r="E65" s="98"/>
-      <c r="F65" s="99"/>
-      <c r="G65" s="99"/>
-      <c r="H65" s="100"/>
-      <c r="I65" s="101"/>
-      <c r="J65" s="101"/>
-      <c r="K65" s="101"/>
-      <c r="L65" s="102"/>
-      <c r="M65" s="102"/>
-      <c r="N65" s="102"/>
-      <c r="O65" s="103"/>
-      <c r="P65" s="102"/>
-      <c r="Q65" s="104"/>
-      <c r="R65" s="104"/>
-      <c r="S65" s="104"/>
-      <c r="T65" s="104"/>
-      <c r="U65" s="104"/>
-      <c r="V65" s="104"/>
-      <c r="W65" s="104"/>
-      <c r="X65" s="104"/>
-      <c r="Y65" s="104"/>
-      <c r="Z65" s="104"/>
-      <c r="AA65" s="104"/>
-      <c r="AB65" s="104"/>
-      <c r="AC65" s="104"/>
-      <c r="AD65" s="104"/>
+    <row r="62" spans="1:31" ht="15" customHeight="1">
+      <c r="C62" s="94"/>
+      <c r="D62" s="95"/>
+      <c r="E62" s="96"/>
+      <c r="F62" s="97"/>
+      <c r="G62" s="97"/>
+      <c r="H62" s="98"/>
+      <c r="I62" s="99"/>
+      <c r="J62" s="99"/>
+      <c r="K62" s="99"/>
+      <c r="L62" s="100"/>
+      <c r="M62" s="100"/>
+      <c r="N62" s="100"/>
+      <c r="O62" s="101"/>
+      <c r="P62" s="100"/>
+      <c r="Q62" s="102"/>
+      <c r="R62" s="102"/>
+      <c r="S62" s="102"/>
+      <c r="T62" s="102"/>
+      <c r="U62" s="102"/>
+      <c r="V62" s="102"/>
+      <c r="W62" s="102"/>
+      <c r="X62" s="102"/>
+      <c r="Y62" s="102"/>
+      <c r="Z62" s="102"/>
+      <c r="AA62" s="102"/>
+      <c r="AB62" s="102"/>
+      <c r="AC62" s="102"/>
+      <c r="AD62" s="102"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
+  <mergeCells count="3">
     <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C36:D36"/>
   </mergeCells>
-  <conditionalFormatting sqref="I65:K65">
+  <conditionalFormatting sqref="I62:K62">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5770,15 +5564,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K58">
-    <cfRule type="cellIs" dxfId="89" priority="1" operator="equal">
+  <conditionalFormatting sqref="K55">
+    <cfRule type="cellIs" dxfId="82" priority="1" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="6" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I58">
+  <conditionalFormatting sqref="I55">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5788,22 +5582,22 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F65">
-    <cfRule type="cellIs" dxfId="87" priority="10" operator="equal">
+  <conditionalFormatting sqref="F62">
+    <cfRule type="cellIs" dxfId="80" priority="10" operator="equal">
       <formula>"Definition"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G65">
-    <cfRule type="cellIs" dxfId="86" priority="9" operator="equal">
+  <conditionalFormatting sqref="G62">
+    <cfRule type="cellIs" dxfId="79" priority="9" operator="equal">
       <formula>"Note"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E58">
-    <cfRule type="cellIs" dxfId="85" priority="8" operator="equal">
+  <conditionalFormatting sqref="E55">
+    <cfRule type="cellIs" dxfId="78" priority="8" operator="equal">
       <formula>"Dataset Description"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F12:F15">
+  <conditionalFormatting sqref="F12:F14">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5813,17 +5607,17 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C65">
-    <cfRule type="cellIs" dxfId="84" priority="4" operator="equal">
+  <conditionalFormatting sqref="C62">
+    <cfRule type="cellIs" dxfId="77" priority="4" operator="equal">
       <formula>"Link"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C58">
-    <cfRule type="cellIs" dxfId="83" priority="3" operator="equal">
+  <conditionalFormatting sqref="C55">
+    <cfRule type="cellIs" dxfId="76" priority="3" operator="equal">
       <formula>"Link"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J58">
+  <conditionalFormatting sqref="J55">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5834,17 +5628,16 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="D62" location="'Country Stats'!A1" display="Country Stats" xr:uid="{37F97D7D-6476-49BF-9118-0DA3787A2751}"/>
+    <hyperlink ref="D59" location="'Country Stats'!A1" display="Country Stats" xr:uid="{37F97D7D-6476-49BF-9118-0DA3787A2751}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <tableParts count="6">
+  <tableParts count="5">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
     <tablePart r:id="rId6"/>
-    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5855,16 +5648,16 @@
     <tabColor rgb="FF131313"/>
   </sheetPr>
   <dimension ref="A1:H83"/>
-  <sheetFormatPr defaultColWidth="15.6640625" defaultRowHeight="15" customHeight="1" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="15.7109375" defaultRowHeight="15" customHeight="1" outlineLevelRow="2"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="8.33203125" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" customWidth="1"/>
-    <col min="5" max="6" width="27.6640625" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="6" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19.95" hidden="1" customHeight="1">
+    <row r="1" spans="1:8" ht="19.899999999999999" hidden="1" customHeight="1">
       <c r="B1" s="13"/>
       <c r="C1" s="14"/>
       <c r="D1" s="14" t="s">
@@ -5875,96 +5668,96 @@
       <c r="G1" s="14"/>
       <c r="H1" s="14"/>
     </row>
-    <row r="2" spans="1:8" s="76" customFormat="1" ht="4.95" customHeight="1">
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
-    </row>
-    <row r="3" spans="1:8" ht="14.4" customHeight="1">
-      <c r="B3" s="86" t="str">
+    <row r="2" spans="1:8" s="75" customFormat="1" ht="4.9000000000000004" customHeight="1">
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="76"/>
+    </row>
+    <row r="3" spans="1:8" ht="14.45" customHeight="1">
+      <c r="B3" s="84" t="str">
         <f ca="1">HYPERLINK("#" &amp; CELL("address", _xlfn.XLOOKUP(Name,tbl_DfOverview[Dataframe],tbl_DfOverview[_],tbl_DfOverview[[#Headers],[_]])), "Overview ↩")</f>
         <v>Overview ↩</v>
       </c>
-      <c r="C3" s="86"/>
-    </row>
-    <row r="4" spans="1:8" ht="4.95" customHeight="1">
-      <c r="B4" s="70"/>
+      <c r="C3" s="84"/>
+    </row>
+    <row r="4" spans="1:8" ht="4.9000000000000004" customHeight="1">
+      <c r="B4" s="69"/>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1">
-      <c r="B5" s="111" t="e" vm="1">
+      <c r="B5" s="109" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C5" s="79" t="s">
-        <v>102</v>
+      <c r="C5" s="78" t="s">
+        <v>99</v>
       </c>
       <c r="D5" s="22"/>
     </row>
-    <row r="6" spans="1:8" ht="10.199999999999999" customHeight="1"/>
-    <row r="7" spans="1:8" ht="14.4">
-      <c r="A7" s="68"/>
-      <c r="B7" s="88" t="s">
-        <v>63</v>
+    <row r="6" spans="1:8" ht="10.15" customHeight="1"/>
+    <row r="7" spans="1:8">
+      <c r="A7" s="67"/>
+      <c r="B7" s="86" t="s">
+        <v>61</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="10.199999999999999" customHeight="1">
-      <c r="A8" s="68"/>
-    </row>
-    <row r="9" spans="1:8" ht="49.95" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A9" s="68"/>
-      <c r="D9" s="73" t="s">
+    <row r="8" spans="1:8" ht="10.15" customHeight="1">
+      <c r="A8" s="67"/>
+    </row>
+    <row r="9" spans="1:8" ht="49.9" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A9" s="67"/>
+      <c r="D9" s="72" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="74"/>
-    </row>
-    <row r="10" spans="1:8" ht="14.4" hidden="1" outlineLevel="1">
-      <c r="A10" s="68"/>
+      <c r="E9" s="73"/>
+    </row>
+    <row r="10" spans="1:8" hidden="1" outlineLevel="1">
+      <c r="A10" s="67"/>
     </row>
     <row r="11" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A11" s="68"/>
+      <c r="A11" s="67"/>
       <c r="C11" s="21" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="32"/>
     </row>
     <row r="12" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A12" s="68"/>
+      <c r="A12" s="67"/>
       <c r="C12" s="3" t="s">
         <v>48</v>
       </c>
       <c r="D12" s="24"/>
     </row>
     <row r="13" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A13" s="68"/>
+      <c r="A13" s="67"/>
       <c r="C13" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="24"/>
     </row>
     <row r="14" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A14" s="68"/>
+      <c r="A14" s="67"/>
       <c r="C14" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D14" s="30"/>
     </row>
     <row r="15" spans="1:8" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A15" s="68"/>
+      <c r="A15" s="67"/>
       <c r="C15" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D15" s="31"/>
     </row>
-    <row r="16" spans="1:8" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A16" s="68"/>
-    </row>
-    <row r="17" spans="1:6" ht="34.950000000000003" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A17" s="68"/>
+    <row r="16" spans="1:8" ht="10.15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A16" s="67"/>
+    </row>
+    <row r="17" spans="1:6" ht="34.9" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A17" s="67"/>
       <c r="C17" s="21" t="s">
         <v>2</v>
       </c>
@@ -5978,10 +5771,10 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="A18" s="68"/>
-    </row>
-    <row r="19" spans="1:6" ht="34.950000000000003" hidden="1" customHeight="1" outlineLevel="1">
+    <row r="18" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="A18" s="67"/>
+    </row>
+    <row r="19" spans="1:6" ht="34.9" hidden="1" customHeight="1" outlineLevel="1">
       <c r="C19" s="21" t="s">
         <v>3</v>
       </c>
@@ -5995,31 +5788,31 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="1"/>
+    <row r="20" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="1"/>
     <row r="21" spans="1:6" s="23" customFormat="1" ht="30" customHeight="1" collapsed="1">
-      <c r="B21" s="59"/>
-      <c r="C21" s="59" t="s">
+      <c r="B21" s="58"/>
+      <c r="C21" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="60"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="60"/>
-    </row>
-    <row r="22" spans="1:6" ht="10.199999999999999" customHeight="1"/>
-    <row r="23" spans="1:6" ht="14.4" outlineLevel="1">
-      <c r="A23" s="68"/>
-      <c r="B23" s="88" t="s">
-        <v>63</v>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="59"/>
+    </row>
+    <row r="22" spans="1:6" ht="10.15" customHeight="1"/>
+    <row r="23" spans="1:6" outlineLevel="1">
+      <c r="A23" s="67"/>
+      <c r="B23" s="86" t="s">
+        <v>61</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="10.199999999999999" customHeight="1" outlineLevel="1">
-      <c r="A24" s="68"/>
+    <row r="24" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+      <c r="A24" s="67"/>
     </row>
     <row r="25" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A25" s="68"/>
+      <c r="A25" s="67"/>
       <c r="C25" s="19" t="s">
         <v>8</v>
       </c>
@@ -6028,7 +5821,7 @@
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A26" s="68"/>
+      <c r="A26" s="67"/>
       <c r="C26" s="3" t="s">
         <v>9</v>
       </c>
@@ -6037,7 +5830,7 @@
       <c r="F26" s="10"/>
     </row>
     <row r="27" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A27" s="68"/>
+      <c r="A27" s="67"/>
       <c r="C27" s="18" t="s">
         <v>10</v>
       </c>
@@ -6046,7 +5839,7 @@
       <c r="F27" s="10"/>
     </row>
     <row r="28" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A28" s="68"/>
+      <c r="A28" s="67"/>
       <c r="C28" s="18" t="s">
         <v>11</v>
       </c>
@@ -6055,7 +5848,7 @@
       <c r="F28" s="10"/>
     </row>
     <row r="29" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A29" s="68"/>
+      <c r="A29" s="67"/>
       <c r="C29" s="18" t="s">
         <v>12</v>
       </c>
@@ -6064,7 +5857,7 @@
       <c r="F29" s="11"/>
     </row>
     <row r="30" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A30" s="68"/>
+      <c r="A30" s="67"/>
       <c r="C30" s="18" t="s">
         <v>13</v>
       </c>
@@ -6073,7 +5866,7 @@
       <c r="F30" s="11"/>
     </row>
     <row r="31" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A31" s="68"/>
+      <c r="A31" s="67"/>
       <c r="C31" s="19" t="s">
         <v>14</v>
       </c>
@@ -6082,7 +5875,7 @@
       <c r="F31" s="11"/>
     </row>
     <row r="32" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A32" s="68"/>
+      <c r="A32" s="67"/>
       <c r="C32" s="3" t="s">
         <v>15</v>
       </c>
@@ -6090,25 +5883,25 @@
       <c r="E32" s="11"/>
       <c r="F32" s="11"/>
     </row>
-    <row r="33" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A33" s="68"/>
-    </row>
-    <row r="34" spans="1:6" ht="124.95" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="35" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="36" spans="1:6" ht="14.4" outlineLevel="1" collapsed="1">
-      <c r="A36" s="68"/>
-      <c r="B36" s="88" t="s">
-        <v>63</v>
+    <row r="33" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A33" s="67"/>
+    </row>
+    <row r="34" spans="1:6" ht="124.9" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="35" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="36" spans="1:6" outlineLevel="1" collapsed="1">
+      <c r="A36" s="67"/>
+      <c r="B36" s="86" t="s">
+        <v>61</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="10.199999999999999" customHeight="1" outlineLevel="1">
-      <c r="A37" s="68"/>
+    <row r="37" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+      <c r="A37" s="67"/>
     </row>
     <row r="38" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A38" s="68"/>
+      <c r="A38" s="67"/>
       <c r="C38" s="3" t="s">
         <v>17</v>
       </c>
@@ -6117,7 +5910,7 @@
       <c r="F38" s="12"/>
     </row>
     <row r="39" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A39" s="68"/>
+      <c r="A39" s="67"/>
       <c r="C39" s="18" t="s">
         <v>18</v>
       </c>
@@ -6126,7 +5919,7 @@
       <c r="F39" s="12"/>
     </row>
     <row r="40" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A40" s="68"/>
+      <c r="A40" s="67"/>
       <c r="C40" s="18" t="s">
         <v>19</v>
       </c>
@@ -6135,7 +5928,7 @@
       <c r="F40" s="12"/>
     </row>
     <row r="41" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A41" s="68"/>
+      <c r="A41" s="67"/>
       <c r="C41" s="3" t="s">
         <v>20</v>
       </c>
@@ -6144,7 +5937,7 @@
       <c r="F41" s="12"/>
     </row>
     <row r="42" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A42" s="68"/>
+      <c r="A42" s="67"/>
       <c r="C42" s="20" t="s">
         <v>21</v>
       </c>
@@ -6152,25 +5945,25 @@
       <c r="E42" s="12"/>
       <c r="F42" s="12"/>
     </row>
-    <row r="43" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A43" s="68"/>
+    <row r="43" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2">
+      <c r="A43" s="67"/>
     </row>
     <row r="44" spans="1:6" ht="150" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="45" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="46" spans="1:6" ht="14.4" outlineLevel="1" collapsed="1">
-      <c r="A46" s="68"/>
-      <c r="B46" s="88" t="s">
-        <v>63</v>
+    <row r="45" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="46" spans="1:6" outlineLevel="1" collapsed="1">
+      <c r="A46" s="67"/>
+      <c r="B46" s="86" t="s">
+        <v>61</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="10.050000000000001" customHeight="1" outlineLevel="1">
-      <c r="A47" s="68"/>
+    <row r="47" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+      <c r="A47" s="67"/>
     </row>
     <row r="48" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A48" s="68"/>
+      <c r="A48" s="67"/>
       <c r="C48" s="3" t="s">
         <v>23</v>
       </c>
@@ -6179,7 +5972,7 @@
       <c r="F48" s="12"/>
     </row>
     <row r="49" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A49" s="68"/>
+      <c r="A49" s="67"/>
       <c r="C49" s="18">
         <v>0.05</v>
       </c>
@@ -6188,7 +5981,7 @@
       <c r="F49" s="12"/>
     </row>
     <row r="50" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A50" s="68"/>
+      <c r="A50" s="67"/>
       <c r="C50" s="19">
         <v>0.25</v>
       </c>
@@ -6197,7 +5990,7 @@
       <c r="F50" s="12"/>
     </row>
     <row r="51" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A51" s="68"/>
+      <c r="A51" s="67"/>
       <c r="C51" s="3">
         <v>0.5</v>
       </c>
@@ -6206,7 +5999,7 @@
       <c r="F51" s="12"/>
     </row>
     <row r="52" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A52" s="68"/>
+      <c r="A52" s="67"/>
       <c r="C52" s="18">
         <v>0.75</v>
       </c>
@@ -6215,7 +6008,7 @@
       <c r="F52" s="12"/>
     </row>
     <row r="53" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A53" s="68"/>
+      <c r="A53" s="67"/>
       <c r="C53" s="18">
         <v>0.95</v>
       </c>
@@ -6224,7 +6017,7 @@
       <c r="F53" s="12"/>
     </row>
     <row r="54" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A54" s="68"/>
+      <c r="A54" s="67"/>
       <c r="C54" s="3" t="s">
         <v>24</v>
       </c>
@@ -6233,7 +6026,7 @@
       <c r="F54" s="12"/>
     </row>
     <row r="55" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A55" s="68"/>
+      <c r="A55" s="67"/>
       <c r="C55" s="18" t="s">
         <v>25</v>
       </c>
@@ -6249,21 +6042,21 @@
       <c r="E56" s="12"/>
       <c r="F56" s="12"/>
     </row>
-    <row r="57" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="58" spans="1:6" ht="14.4" outlineLevel="1" collapsed="1">
-      <c r="A58" s="68"/>
-      <c r="B58" s="88" t="s">
-        <v>63</v>
+    <row r="57" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="58" spans="1:6" outlineLevel="1" collapsed="1">
+      <c r="A58" s="67"/>
+      <c r="B58" s="86" t="s">
+        <v>61</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="10.050000000000001" customHeight="1" outlineLevel="1">
-      <c r="A59" s="68"/>
+    <row r="59" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+      <c r="A59" s="67"/>
     </row>
     <row r="60" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A60" s="68"/>
+      <c r="A60" s="67"/>
       <c r="C60" s="3" t="s">
         <v>28</v>
       </c>
@@ -6278,7 +6071,7 @@
       </c>
     </row>
     <row r="61" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A61" s="68"/>
+      <c r="A61" s="67"/>
       <c r="C61" s="18" t="s">
         <v>29</v>
       </c>
@@ -6293,7 +6086,7 @@
       </c>
     </row>
     <row r="62" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A62" s="68"/>
+      <c r="A62" s="67"/>
       <c r="C62" s="18" t="s">
         <v>30</v>
       </c>
@@ -6308,7 +6101,7 @@
       </c>
     </row>
     <row r="63" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A63" s="68"/>
+      <c r="A63" s="67"/>
       <c r="C63" s="18" t="s">
         <v>31</v>
       </c>
@@ -6323,7 +6116,7 @@
       </c>
     </row>
     <row r="64" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A64" s="68"/>
+      <c r="A64" s="67"/>
       <c r="C64" s="3" t="s">
         <v>32</v>
       </c>
@@ -6338,7 +6131,7 @@
       </c>
     </row>
     <row r="65" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A65" s="68"/>
+      <c r="A65" s="67"/>
       <c r="C65" s="18" t="s">
         <v>33</v>
       </c>
@@ -6353,7 +6146,7 @@
       </c>
     </row>
     <row r="66" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A66" s="68"/>
+      <c r="A66" s="67"/>
       <c r="C66" s="18" t="s">
         <v>34</v>
       </c>
@@ -6381,21 +6174,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="2"/>
-    <row r="69" spans="1:6" ht="14.4" outlineLevel="1" collapsed="1">
-      <c r="A69" s="68"/>
-      <c r="B69" s="88" t="s">
-        <v>63</v>
+    <row r="68" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
+    <row r="69" spans="1:6" outlineLevel="1" collapsed="1">
+      <c r="A69" s="67"/>
+      <c r="B69" s="86" t="s">
+        <v>61</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="10.050000000000001" customHeight="1" outlineLevel="1">
-      <c r="A70" s="68"/>
+    <row r="70" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+      <c r="A70" s="67"/>
     </row>
     <row r="71" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A71" s="68"/>
+      <c r="A71" s="67"/>
       <c r="C71" s="3" t="str">
         <f>IF(COUNTIF(FieldList1, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C60)," ","_") &amp;" = ")</f>
         <v/>
@@ -6406,7 +6199,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A72" s="68"/>
+      <c r="A72" s="67"/>
       <c r="C72" s="17" t="str">
         <f>IF(COUNTIF(FieldList2, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C61)," ","_")&amp;" = ")</f>
         <v/>
@@ -6417,7 +6210,7 @@
       </c>
     </row>
     <row r="73" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A73" s="68"/>
+      <c r="A73" s="67"/>
       <c r="C73" s="17" t="str">
         <f>IF(COUNTIF(FieldList3, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C62)," ","_")&amp;" = ")</f>
         <v/>
@@ -6428,7 +6221,7 @@
       </c>
     </row>
     <row r="74" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A74" s="68"/>
+      <c r="A74" s="67"/>
       <c r="C74" s="17" t="str">
         <f>IF(COUNTIF(FieldList4, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C63)," ","_")&amp;" = ")</f>
         <v/>
@@ -6439,7 +6232,7 @@
       </c>
     </row>
     <row r="75" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A75" s="68"/>
+      <c r="A75" s="67"/>
       <c r="C75" s="17" t="str">
         <f>IF(COUNTIF(FieldList5, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C64)," ","_")&amp;" = ")</f>
         <v/>
@@ -6450,7 +6243,7 @@
       </c>
     </row>
     <row r="76" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A76" s="68"/>
+      <c r="A76" s="67"/>
       <c r="C76" s="17" t="str">
         <f>IF(COUNTIF(FieldList6, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C65)," ","_")&amp;" = ")</f>
         <v/>
@@ -6461,7 +6254,7 @@
       </c>
     </row>
     <row r="77" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A77" s="68"/>
+      <c r="A77" s="67"/>
       <c r="C77" s="16" t="str">
         <f>IF(COUNTIF(FieldList7, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C66)," ","_")&amp;" = ")</f>
         <v/>
@@ -6472,7 +6265,7 @@
       </c>
     </row>
     <row r="78" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
-      <c r="A78" s="68"/>
+      <c r="A78" s="67"/>
       <c r="C78" s="3" t="str">
         <f>IF(COUNTIF(FieldList8, "&lt;&gt;FALSE") = 0,"",SUBSTITUTE(LOWER(C67)," ","_")&amp;" = ")</f>
         <v/>
@@ -6492,36 +6285,36 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="10.199999999999999" hidden="1" customHeight="1" outlineLevel="1" collapsed="1"/>
+    <row r="80" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="1" collapsed="1"/>
     <row r="81" spans="3:6" ht="30" customHeight="1">
-      <c r="C81" s="63" t="s">
+      <c r="C81" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="D81" s="61" t="s">
-        <v>95</v>
-      </c>
-      <c r="E81" s="61" t="s">
+      <c r="D81" s="60" t="s">
+        <v>93</v>
+      </c>
+      <c r="E81" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="F81" s="61" t="s">
-        <v>96</v>
+      <c r="F81" s="60" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="82" spans="3:6" ht="15" customHeight="1">
-      <c r="C82" s="64" t="b">
+      <c r="C82" s="63" t="b">
         <v>0</v>
       </c>
-      <c r="D82" s="62"/>
-      <c r="E82" s="80"/>
-      <c r="F82" s="62"/>
+      <c r="D82" s="61"/>
+      <c r="E82" s="79"/>
+      <c r="F82" s="61"/>
     </row>
     <row r="83" spans="3:6" ht="15" customHeight="1">
-      <c r="C83" s="71" t="b">
+      <c r="C83" s="70" t="b">
         <v>0</v>
       </c>
-      <c r="D83" s="62"/>
-      <c r="E83" s="80"/>
-      <c r="F83" s="62"/>
+      <c r="D83" s="61"/>
+      <c r="E83" s="79"/>
+      <c r="F83" s="61"/>
     </row>
   </sheetData>
   <phoneticPr fontId="24" type="noConversion"/>

</xml_diff>

<commit_message>
Added theme setting/VBA toggling to CLI, new readme sections
Added theme setting/VBA toggling to CLI, new readme sections

Add CLI/xleda for non developers sections to readme
</commit_message>
<xml_diff>
--- a/src/xleda/xleda_template.xlsx
+++ b/src/xleda/xleda_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8FA3A98-AC7F-49B5-BE3A-E5583C25AD62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4919C7DC-91C5-4547-B1D5-9BD11905218F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
@@ -18,21 +18,21 @@
     <sheet name="Field Analysis" sheetId="25" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="Back">Overview!$D$54</definedName>
+    <definedName name="Back">Overview!$D$57</definedName>
     <definedName name="Compiled_Lists" localSheetId="2">'Field Analysis'!$C$71:$C$80</definedName>
     <definedName name="Composition" localSheetId="2">'Field Analysis'!$C$25:$C$35</definedName>
     <definedName name="CompositionTable" localSheetId="2">'Field Analysis'!$D$34</definedName>
     <definedName name="DarkHeader" localSheetId="2">'Field Analysis'!$D$81</definedName>
     <definedName name="Data_Description" localSheetId="2">'Field Analysis'!$C$9:$C$20</definedName>
-    <definedName name="Dataframes">Overview!$C$54:$C$57</definedName>
-    <definedName name="Debug" localSheetId="1">Overview!$D$9:$E$51</definedName>
+    <definedName name="Dataframes">Overview!$C$57:$C$60</definedName>
+    <definedName name="Debug" localSheetId="1">Overview!$D$9:$E$54</definedName>
     <definedName name="DebugToggle" localSheetId="1">Overview!$B$6</definedName>
     <definedName name="Definitions" localSheetId="2">'Field Analysis'!$D$17:$F$17</definedName>
     <definedName name="Description" localSheetId="2">'Field Analysis'!$D$9</definedName>
     <definedName name="Dimensions" localSheetId="2">'Field Analysis'!$D$11</definedName>
     <definedName name="Field_Analysis" localSheetId="2">'Field Analysis'!$D$22:$D$80</definedName>
     <definedName name="Field_Lists" localSheetId="2">'Field Analysis'!$C$60:$C$68</definedName>
-    <definedName name="Field_Overview">Overview!$E$61:$E$62</definedName>
+    <definedName name="Field_Overview">Overview!$E$64:$E$65</definedName>
     <definedName name="FieldList1" localSheetId="2">'Field Analysis'!$D$60:$F$60</definedName>
     <definedName name="FieldList2" localSheetId="2">'Field Analysis'!$D$61:$F$61</definedName>
     <definedName name="FieldList3" localSheetId="2">'Field Analysis'!$D$62:$F$62</definedName>
@@ -43,7 +43,7 @@
     <definedName name="FieldList8" localSheetId="2">'Field Analysis'!$D$67:$F$67</definedName>
     <definedName name="FieldLists" localSheetId="2">'Field Analysis'!$C$60:$F$67</definedName>
     <definedName name="FieldRange" localSheetId="2">'Field Analysis'!$D$81:$F$81</definedName>
-    <definedName name="Fields">Overview!$C$61:$C$62</definedName>
+    <definedName name="Fields">Overview!$C$64:$C$65</definedName>
     <definedName name="FormatRange" localSheetId="2">'Field Analysis'!$F:$F</definedName>
     <definedName name="Headers" localSheetId="2">'Field Analysis'!$D$21:$F$21</definedName>
     <definedName name="Headers_Start" localSheetId="2">'Field Analysis'!$D$21</definedName>
@@ -58,7 +58,7 @@
     <definedName name="SinglePlot" localSheetId="0">SinglePlot!$C$10</definedName>
     <definedName name="Summary_Stats" localSheetId="2">'Field Analysis'!$C$38:$C$45</definedName>
     <definedName name="Theme" localSheetId="2">'Field Analysis'!$B$21:$F$21</definedName>
-    <definedName name="Theme" localSheetId="1">Overview!$E$61:$AD$61</definedName>
+    <definedName name="Theme" localSheetId="1">Overview!$E$64:$AD$64</definedName>
     <definedName name="Theme" localSheetId="0">SinglePlot!$B$8:$P$8</definedName>
     <definedName name="Toggles" localSheetId="2">'Field Analysis'!$B$7,'Field Analysis'!$B$23,'Field Analysis'!$B$36,'Field Analysis'!$B$46,'Field Analysis'!$B$58,'Field Analysis'!$B$69</definedName>
     <definedName name="TopToggle" localSheetId="2">'Field Analysis'!$B$5</definedName>
@@ -125,7 +125,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="108">
   <si>
     <t>Warning</t>
   </si>
@@ -443,6 +443,12 @@
   </si>
   <si>
     <t>data argument</t>
+  </si>
+  <si>
+    <t>xleda Documentation:</t>
+  </si>
+  <si>
+    <t>https://github.com/InfoDesigner/xleda/</t>
   </si>
 </sst>
 </file>
@@ -705,13 +711,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="4"/>
-      <color theme="1" tint="0.39997558519241921"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <i/>
       <sz val="6"/>
@@ -723,6 +722,15 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1" tint="0.39997558519241921"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="8"/>
       <color theme="1" tint="0.39997558519241921"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1063,7 +1071,7 @@
     </xf>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" textRotation="180"/>
@@ -1287,10 +1295,7 @@
     <xf numFmtId="3" fontId="10" fillId="8" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -1373,13 +1378,13 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="35" fillId="5" borderId="16" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="34" fillId="5" borderId="16" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="35" fillId="5" borderId="19" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="3" fontId="34" fillId="5" borderId="19" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="35" fillId="5" borderId="17" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="3" fontId="34" fillId="5" borderId="17" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="10" fillId="2" borderId="18" xfId="7" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1387,6 +1392,13 @@
     </xf>
     <xf numFmtId="3" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="32" fillId="2" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -4353,7 +4365,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E2133564-163D-4CB0-A97C-9358270F5F9C}" name="tbl_debug_section" displayName="tbl_debug_section" ref="D11:F14" totalsRowShown="0" headerRowDxfId="75" dataDxfId="73" headerRowBorderDxfId="74" tableBorderDxfId="72" totalsRowBorderDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E2133564-163D-4CB0-A97C-9358270F5F9C}" name="tbl_debug_section" displayName="tbl_debug_section" ref="D14:F17" totalsRowShown="0" headerRowDxfId="75" dataDxfId="73" headerRowBorderDxfId="74" tableBorderDxfId="72" totalsRowBorderDxfId="71">
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5EB43B6F-4FF7-4D4C-8202-BD94842B8017}" name="Production Section" dataDxfId="70" dataCellStyle="DarkHeader"/>
     <tableColumn id="2" xr3:uid="{71F0A434-8F03-4CF9-987C-D6F88D936E0A}" name="Production Time in Seconds" dataDxfId="69"/>
@@ -4364,7 +4376,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FABCC19D-29F4-4A1C-9C2C-61132A93E32D}" name="tbl_debug_environment" displayName="tbl_debug_environment" ref="D19:E33" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FABCC19D-29F4-4A1C-9C2C-61132A93E32D}" name="tbl_debug_environment" displayName="tbl_debug_environment" ref="D22:E36" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{6A891059-3C09-438F-9AB9-42F8BA5B3379}" name="Environment Variable" dataDxfId="63" dataCellStyle="DarkHeader"/>
     <tableColumn id="2" xr3:uid="{D9E0C91D-D549-4194-8575-1343B51883A7}" name="Value" dataDxfId="62"/>
@@ -4374,7 +4386,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{88D10CD5-62A0-484D-A455-84E38CB47746}" name="tbl_debug_config" displayName="tbl_debug_config" ref="D38:E50" totalsRowShown="0" headerRowDxfId="61" headerRowBorderDxfId="60" tableBorderDxfId="59" totalsRowBorderDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{88D10CD5-62A0-484D-A455-84E38CB47746}" name="tbl_debug_config" displayName="tbl_debug_config" ref="D41:E53" totalsRowShown="0" headerRowDxfId="61" headerRowBorderDxfId="60" tableBorderDxfId="59" totalsRowBorderDxfId="58">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{BAFB02A5-6AA3-46EF-A3FA-1FC44F32BBF4}" name="Input Argument" dataDxfId="57" dataCellStyle="DarkHeader"/>
     <tableColumn id="2" xr3:uid="{402A365F-6164-4790-9B23-3CC27E2F5642}" name="Value" dataDxfId="56" dataCellStyle="DarkHeader"/>
@@ -4384,7 +4396,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AFE650AA-A988-4967-9BF1-5CBBD5AE48A6}" name="tbl_FieldOverview" displayName="tbl_FieldOverview" ref="C61:AD62" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AFE650AA-A988-4967-9BF1-5CBBD5AE48A6}" name="tbl_FieldOverview" displayName="tbl_FieldOverview" ref="C64:AD65" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54">
   <tableColumns count="28">
     <tableColumn id="1" xr3:uid="{BFB84B7E-8B25-47B3-90FE-AC7BFBAF30EB}" name="_" dataDxfId="52" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{50D3F477-2874-418A-8431-FEC88B724332}" name="Dataframe" dataDxfId="51"/>
@@ -4420,7 +4432,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B62C177-35BB-4328-A5E9-CE2D42C175A6}" name="tbl_DfOverview" displayName="tbl_DfOverview" ref="C54:K55" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B62C177-35BB-4328-A5E9-CE2D42C175A6}" name="tbl_DfOverview" displayName="tbl_DfOverview" ref="C57:K58" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{95AE6ED1-2225-487F-9D3B-3E94D426571D}" name="_" dataDxfId="21" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{19718F20-2450-421A-9215-32A414225B3E}" name="Dataframe" dataDxfId="20" dataCellStyle="Hyperlink"/>
@@ -4799,17 +4811,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="4.9000000000000004" customHeight="1"/>
-    <row r="2" spans="2:16" ht="14.45" customHeight="1">
-      <c r="B2" s="84" t="s">
+    <row r="2" spans="2:16" ht="20.100000000000001" customHeight="1">
+      <c r="B2" s="119" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="84"/>
+      <c r="D2" s="83"/>
     </row>
     <row r="3" spans="2:16" ht="10.15" customHeight="1">
       <c r="B3" s="77"/>
     </row>
     <row r="4" spans="2:16" ht="30" customHeight="1">
-      <c r="B4" s="109" t="e" vm="1">
+      <c r="B4" s="108" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="C4" s="53" t="s">
@@ -4879,7 +4891,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:AE62"/>
+  <dimension ref="A1:AE65"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -4893,7 +4905,7 @@
     <col min="21" max="30" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="85" customFormat="1" ht="4.9000000000000004" customHeight="1">
+    <row r="1" spans="1:28" s="84" customFormat="1" ht="4.9000000000000004" customHeight="1">
       <c r="H1"/>
       <c r="I1"/>
       <c r="J1"/>
@@ -4901,14 +4913,14 @@
     <row r="2" spans="1:28" ht="14.45" customHeight="1">
       <c r="A2" s="71"/>
     </row>
-    <row r="3" spans="1:28" s="85" customFormat="1" ht="10.15" customHeight="1">
+    <row r="3" spans="1:28" s="84" customFormat="1" ht="10.15" customHeight="1">
       <c r="A3" s="71"/>
       <c r="H3"/>
       <c r="I3"/>
       <c r="J3"/>
     </row>
     <row r="4" spans="1:28" ht="30" customHeight="1">
-      <c r="B4" s="110" t="e" vm="1">
+      <c r="B4" s="109" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="C4" s="53" t="s">
@@ -4917,15 +4929,15 @@
       <c r="D4" s="74"/>
       <c r="AB4" s="4"/>
     </row>
-    <row r="5" spans="1:28" ht="10.15" customHeight="1">
+    <row r="5" spans="1:28" ht="20.100000000000001" customHeight="1">
       <c r="C5" s="53"/>
       <c r="AB5" s="4"/>
     </row>
     <row r="6" spans="1:28" ht="15" customHeight="1">
-      <c r="B6" s="83" t="s">
+      <c r="B6" s="118" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="84" t="s">
+      <c r="C6" s="119" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="51"/>
@@ -4942,236 +4954,222 @@
       <c r="G7" s="43"/>
       <c r="K7" s="43"/>
     </row>
-    <row r="8" spans="1:28" ht="15" customHeight="1">
+    <row r="8" spans="1:28" ht="20.100000000000001" customHeight="1">
       <c r="C8" s="43"/>
       <c r="D8" s="43"/>
       <c r="E8" s="43"/>
       <c r="F8" s="43"/>
-      <c r="G8" s="111"/>
+      <c r="G8" s="110"/>
       <c r="K8" s="43"/>
     </row>
-    <row r="9" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B9" s="1"/>
-      <c r="C9" s="118" t="s">
+    <row r="9" spans="1:28" s="84" customFormat="1" ht="30" hidden="1" customHeight="1">
+      <c r="C9" s="120" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="120"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="117"/>
+      <c r="K9" s="43"/>
+    </row>
+    <row r="10" spans="1:28" s="84" customFormat="1" ht="15" hidden="1" customHeight="1">
+      <c r="C10" s="43"/>
+      <c r="D10" s="82" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="117"/>
+      <c r="K10" s="43"/>
+    </row>
+    <row r="11" spans="1:28" s="84" customFormat="1" ht="15" hidden="1" customHeight="1">
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="117"/>
+      <c r="K11" s="43"/>
+    </row>
+    <row r="12" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B12" s="1"/>
+      <c r="C12" s="120" t="s">
         <v>97</v>
       </c>
-      <c r="D9" s="118"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="K9" s="43"/>
-    </row>
-    <row r="10" spans="1:28" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-    </row>
-    <row r="11" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B11" s="41"/>
-      <c r="D11" s="113" t="s">
+      <c r="D12" s="120"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="K12" s="43"/>
+    </row>
+    <row r="13" spans="1:28" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
+    </row>
+    <row r="14" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B14" s="41"/>
+      <c r="D14" s="112" t="s">
         <v>56</v>
       </c>
-      <c r="E11" s="115" t="s">
+      <c r="E14" s="114" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="114" t="s">
+      <c r="F14" s="113" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D12" s="116" t="s">
+    <row r="15" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D15" s="115" t="s">
         <v>101</v>
       </c>
-      <c r="E12" s="50"/>
-      <c r="F12" s="49"/>
-    </row>
-    <row r="13" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D13" s="116" t="s">
+      <c r="E15" s="50"/>
+      <c r="F15" s="49"/>
+    </row>
+    <row r="16" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D16" s="115" t="s">
         <v>102</v>
       </c>
-      <c r="E13" s="50"/>
-      <c r="F13" s="49"/>
-    </row>
-    <row r="14" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D14" s="116" t="s">
+      <c r="E16" s="50"/>
+      <c r="F16" s="49"/>
+    </row>
+    <row r="17" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D17" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="E14" s="50"/>
-      <c r="F14" s="49"/>
-    </row>
-    <row r="15" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-    </row>
-    <row r="16" spans="1:28" ht="10.15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="L16" s="38"/>
-    </row>
-    <row r="17" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C17" s="118" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="118"/>
-      <c r="E17" s="80"/>
-      <c r="L17" s="38"/>
-    </row>
-    <row r="18" spans="2:12" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="E17" s="50"/>
+      <c r="F17" s="49"/>
+    </row>
+    <row r="18" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C18" s="43"/>
       <c r="D18" s="43"/>
       <c r="E18" s="43"/>
     </row>
-    <row r="19" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D19" s="113" t="s">
+    <row r="19" spans="2:12" ht="10.15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="L19" s="38"/>
+    </row>
+    <row r="20" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C20" s="120" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="120"/>
+      <c r="E20" s="80"/>
+      <c r="L20" s="38"/>
+    </row>
+    <row r="21" spans="2:12" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+    </row>
+    <row r="22" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D22" s="112" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="114" t="s">
+      <c r="E22" s="113" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="20" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D20" s="44" t="s">
-        <v>62</v>
-      </c>
-      <c r="E20" s="56"/>
-    </row>
-    <row r="21" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D21" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" s="56"/>
-    </row>
-    <row r="22" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D22" s="44" t="s">
-        <v>64</v>
-      </c>
-      <c r="E22" s="56"/>
     </row>
     <row r="23" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D23" s="44" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E23" s="56"/>
     </row>
     <row r="24" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D24" s="44" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E24" s="56"/>
     </row>
     <row r="25" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D25" s="44" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E25" s="56"/>
     </row>
     <row r="26" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D26" s="44" t="s">
-        <v>69</v>
-      </c>
-      <c r="E26" s="57"/>
+        <v>66</v>
+      </c>
+      <c r="E26" s="56"/>
     </row>
     <row r="27" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D27" s="44" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E27" s="56"/>
     </row>
     <row r="28" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B28" s="39"/>
       <c r="D28" s="44" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E28" s="56"/>
     </row>
     <row r="29" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D29" s="44" t="s">
-        <v>72</v>
-      </c>
-      <c r="E29" s="56"/>
+        <v>69</v>
+      </c>
+      <c r="E29" s="57"/>
     </row>
     <row r="30" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D30" s="44" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E30" s="56"/>
     </row>
     <row r="31" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B31" s="39"/>
       <c r="D31" s="44" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E31" s="56"/>
-      <c r="I31" s="81"/>
-      <c r="J31" s="82"/>
-      <c r="K31" s="43"/>
     </row>
     <row r="32" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D32" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="56"/>
+    </row>
+    <row r="33" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D33" s="44" t="s">
+        <v>73</v>
+      </c>
+      <c r="E33" s="56"/>
+    </row>
+    <row r="34" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D34" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="E34" s="56"/>
+      <c r="I34" s="81"/>
+      <c r="J34" s="82"/>
+      <c r="K34" s="43"/>
+    </row>
+    <row r="35" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D35" s="44" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="56"/>
-      <c r="K32" s="43"/>
-    </row>
-    <row r="33" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B33" s="40"/>
-      <c r="C33" s="45"/>
-      <c r="D33" s="44" t="s">
+      <c r="E35" s="56"/>
+      <c r="K35" s="43"/>
+    </row>
+    <row r="36" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B36" s="40"/>
+      <c r="C36" s="45"/>
+      <c r="D36" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="56"/>
-      <c r="K33" s="43"/>
-    </row>
-    <row r="34" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B34" s="40"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="81"/>
-      <c r="E34" s="56"/>
-      <c r="K34" s="43"/>
-    </row>
-    <row r="35" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D35" s="47"/>
-      <c r="E35" s="46"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="43"/>
-      <c r="I35" s="43"/>
-      <c r="J35" s="43"/>
-      <c r="K35" s="43"/>
-      <c r="W35" s="42"/>
-      <c r="Y35" s="38"/>
-    </row>
-    <row r="36" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C36" s="118" t="s">
-        <v>53</v>
-      </c>
-      <c r="D36" s="118"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="43"/>
-      <c r="I36" s="43"/>
-      <c r="J36" s="43"/>
+      <c r="E36" s="56"/>
       <c r="K36" s="43"/>
-      <c r="W36" s="42"/>
-      <c r="Y36" s="38"/>
-    </row>
-    <row r="37" spans="2:25" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="43"/>
-      <c r="I37" s="43"/>
-      <c r="J37" s="43"/>
+    </row>
+    <row r="37" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B37" s="40"/>
+      <c r="C37" s="45"/>
+      <c r="D37" s="81"/>
+      <c r="E37" s="56"/>
       <c r="K37" s="43"/>
-      <c r="W37" s="42"/>
-      <c r="Y37" s="38"/>
-    </row>
-    <row r="38" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D38" s="113" t="s">
-        <v>60</v>
-      </c>
-      <c r="E38" s="114" t="s">
-        <v>55</v>
-      </c>
+    </row>
+    <row r="38" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D38" s="47"/>
+      <c r="E38" s="46"/>
       <c r="F38" s="43"/>
       <c r="G38" s="43"/>
       <c r="H38" s="43"/>
@@ -5181,11 +5179,11 @@
       <c r="W38" s="42"/>
       <c r="Y38" s="38"/>
     </row>
-    <row r="39" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D39" s="48" t="s">
-        <v>103</v>
-      </c>
-      <c r="E39" s="54"/>
+    <row r="39" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C39" s="120" t="s">
+        <v>53</v>
+      </c>
+      <c r="D39" s="120"/>
       <c r="F39" s="43"/>
       <c r="G39" s="43"/>
       <c r="H39" s="43"/>
@@ -5195,11 +5193,9 @@
       <c r="W39" s="42"/>
       <c r="Y39" s="38"/>
     </row>
-    <row r="40" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D40" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="E40" s="55"/>
+    <row r="40" spans="2:25" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
       <c r="F40" s="43"/>
       <c r="G40" s="43"/>
       <c r="H40" s="43"/>
@@ -5209,11 +5205,13 @@
       <c r="W40" s="42"/>
       <c r="Y40" s="38"/>
     </row>
-    <row r="41" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D41" s="64" t="s">
-        <v>105</v>
-      </c>
-      <c r="E41" s="55"/>
+    <row r="41" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D41" s="112" t="s">
+        <v>60</v>
+      </c>
+      <c r="E41" s="113" t="s">
+        <v>55</v>
+      </c>
       <c r="F41" s="43"/>
       <c r="G41" s="43"/>
       <c r="H41" s="43"/>
@@ -5224,10 +5222,10 @@
       <c r="Y41" s="38"/>
     </row>
     <row r="42" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D42" s="64" t="s">
-        <v>77</v>
-      </c>
-      <c r="E42" s="55"/>
+      <c r="D42" s="48" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" s="54"/>
       <c r="F42" s="43"/>
       <c r="G42" s="43"/>
       <c r="H42" s="43"/>
@@ -5238,8 +5236,8 @@
       <c r="Y42" s="38"/>
     </row>
     <row r="43" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D43" s="64" t="s">
-        <v>78</v>
+      <c r="D43" s="44" t="s">
+        <v>104</v>
       </c>
       <c r="E43" s="55"/>
       <c r="F43" s="43"/>
@@ -5253,7 +5251,7 @@
     </row>
     <row r="44" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D44" s="64" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="E44" s="55"/>
       <c r="F44" s="43"/>
@@ -5267,7 +5265,7 @@
     </row>
     <row r="45" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D45" s="64" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E45" s="55"/>
       <c r="F45" s="43"/>
@@ -5281,7 +5279,7 @@
     </row>
     <row r="46" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D46" s="64" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E46" s="55"/>
       <c r="F46" s="43"/>
@@ -5295,7 +5293,7 @@
     </row>
     <row r="47" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D47" s="64" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E47" s="55"/>
       <c r="F47" s="43"/>
@@ -5308,10 +5306,10 @@
       <c r="Y47" s="38"/>
     </row>
     <row r="48" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D48" s="65" t="s">
-        <v>83</v>
-      </c>
-      <c r="E48" s="66"/>
+      <c r="D48" s="64" t="s">
+        <v>80</v>
+      </c>
+      <c r="E48" s="55"/>
       <c r="F48" s="43"/>
       <c r="G48" s="43"/>
       <c r="H48" s="43"/>
@@ -5323,7 +5321,7 @@
     </row>
     <row r="49" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D49" s="64" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E49" s="55"/>
       <c r="F49" s="43"/>
@@ -5336,10 +5334,10 @@
       <c r="Y49" s="38"/>
     </row>
     <row r="50" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D50" s="65" t="s">
-        <v>65</v>
-      </c>
-      <c r="E50" s="66"/>
+      <c r="D50" s="64" t="s">
+        <v>82</v>
+      </c>
+      <c r="E50" s="55"/>
       <c r="F50" s="43"/>
       <c r="G50" s="43"/>
       <c r="H50" s="43"/>
@@ -5350,8 +5348,10 @@
       <c r="Y50" s="38"/>
     </row>
     <row r="51" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D51" s="47"/>
-      <c r="E51" s="46"/>
+      <c r="D51" s="65" t="s">
+        <v>83</v>
+      </c>
+      <c r="E51" s="66"/>
       <c r="F51" s="43"/>
       <c r="G51" s="43"/>
       <c r="H51" s="43"/>
@@ -5361,200 +5361,241 @@
       <c r="W51" s="42"/>
       <c r="Y51" s="38"/>
     </row>
-    <row r="52" spans="1:31" ht="15" customHeight="1" collapsed="1">
-      <c r="A52" s="6"/>
-      <c r="B52" s="68" t="s">
+    <row r="52" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D52" s="64" t="s">
+        <v>84</v>
+      </c>
+      <c r="E52" s="55"/>
+      <c r="F52" s="43"/>
+      <c r="G52" s="43"/>
+      <c r="H52" s="43"/>
+      <c r="I52" s="43"/>
+      <c r="J52" s="43"/>
+      <c r="K52" s="43"/>
+      <c r="W52" s="42"/>
+      <c r="Y52" s="38"/>
+    </row>
+    <row r="53" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D53" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="E53" s="66"/>
+      <c r="F53" s="43"/>
+      <c r="G53" s="43"/>
+      <c r="H53" s="43"/>
+      <c r="I53" s="43"/>
+      <c r="J53" s="43"/>
+      <c r="K53" s="43"/>
+      <c r="W53" s="42"/>
+      <c r="Y53" s="38"/>
+    </row>
+    <row r="54" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D54" s="47"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="43"/>
+      <c r="G54" s="43"/>
+      <c r="H54" s="43"/>
+      <c r="I54" s="43"/>
+      <c r="J54" s="43"/>
+      <c r="K54" s="43"/>
+      <c r="W54" s="42"/>
+      <c r="Y54" s="38"/>
+    </row>
+    <row r="55" spans="1:31" ht="15" customHeight="1" collapsed="1">
+      <c r="A55" s="6"/>
+      <c r="B55" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="C52" s="112" t="s">
+      <c r="C55" s="111" t="s">
         <v>87</v>
       </c>
-      <c r="AB52" s="4"/>
-    </row>
-    <row r="53" spans="1:31" ht="15" customHeight="1">
-      <c r="C53" s="53"/>
-      <c r="AB53" s="4"/>
-    </row>
-    <row r="54" spans="1:31" ht="30" customHeight="1">
-      <c r="C54" s="88" t="s">
+      <c r="AB55" s="4"/>
+    </row>
+    <row r="56" spans="1:31" ht="20.100000000000001" customHeight="1">
+      <c r="C56" s="53"/>
+      <c r="AB56" s="4"/>
+    </row>
+    <row r="57" spans="1:31" ht="30" customHeight="1">
+      <c r="C57" s="87" t="s">
         <v>91</v>
       </c>
-      <c r="D54" s="89" t="s">
+      <c r="D57" s="88" t="s">
         <v>86</v>
       </c>
-      <c r="E54" s="90" t="s">
+      <c r="E57" s="89" t="s">
         <v>100</v>
       </c>
-      <c r="F54" s="87" t="s">
+      <c r="F57" s="86" t="s">
         <v>89</v>
       </c>
-      <c r="G54" s="91" t="s">
+      <c r="G57" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="H54" s="91" t="s">
+      <c r="H57" s="90" t="s">
         <v>48</v>
       </c>
-      <c r="I54" s="91" t="s">
+      <c r="I57" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="J54" s="91" t="s">
+      <c r="J57" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="K54" s="87" t="s">
+      <c r="K57" s="86" t="s">
         <v>98</v>
       </c>
-      <c r="AE54" s="4"/>
-    </row>
-    <row r="55" spans="1:31" ht="15" customHeight="1">
-      <c r="C55" s="94"/>
-      <c r="D55" s="103"/>
-      <c r="E55" s="104"/>
-      <c r="F55" s="117"/>
-      <c r="G55" s="105"/>
-      <c r="H55" s="106"/>
-      <c r="I55" s="107"/>
-      <c r="J55" s="99"/>
-      <c r="K55" s="108"/>
-      <c r="AE55" s="4"/>
-    </row>
-    <row r="57" spans="1:31" ht="15" customHeight="1">
-      <c r="AB57" s="4"/>
+      <c r="AE57" s="4"/>
     </row>
     <row r="58" spans="1:31" ht="15" customHeight="1">
-      <c r="B58" s="68" t="s">
+      <c r="C58" s="93"/>
+      <c r="D58" s="102"/>
+      <c r="E58" s="103"/>
+      <c r="F58" s="116"/>
+      <c r="G58" s="104"/>
+      <c r="H58" s="105"/>
+      <c r="I58" s="106"/>
+      <c r="J58" s="98"/>
+      <c r="K58" s="107"/>
+      <c r="AE58" s="4"/>
+    </row>
+    <row r="60" spans="1:31" ht="15" customHeight="1">
+      <c r="AB60" s="4"/>
+    </row>
+    <row r="61" spans="1:31" ht="15" customHeight="1">
+      <c r="B61" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="C58" s="112" t="s">
+      <c r="C61" s="111" t="s">
         <v>88</v>
       </c>
-      <c r="D58" s="85"/>
-      <c r="AB58" s="4"/>
-    </row>
-    <row r="59" spans="1:31" ht="10.15" customHeight="1"/>
-    <row r="60" spans="1:31" ht="10.15" customHeight="1"/>
-    <row r="61" spans="1:31" ht="30" customHeight="1">
-      <c r="C61" s="88" t="s">
+      <c r="D61" s="84"/>
+      <c r="AB61" s="4"/>
+    </row>
+    <row r="62" spans="1:31" ht="20.100000000000001" customHeight="1"/>
+    <row r="63" spans="1:31" ht="10.15" customHeight="1"/>
+    <row r="64" spans="1:31" ht="30" customHeight="1">
+      <c r="C64" s="87" t="s">
         <v>91</v>
       </c>
-      <c r="D61" s="92" t="s">
+      <c r="D64" s="91" t="s">
         <v>86</v>
       </c>
-      <c r="E61" s="92" t="s">
+      <c r="E64" s="91" t="s">
         <v>39</v>
       </c>
-      <c r="F61" s="92" t="s">
+      <c r="F64" s="91" t="s">
         <v>40</v>
       </c>
-      <c r="G61" s="92" t="s">
+      <c r="G64" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="H61" s="87" t="s">
+      <c r="H64" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="I61" s="87" t="s">
+      <c r="I64" s="86" t="s">
         <v>9</v>
       </c>
-      <c r="J61" s="87" t="s">
+      <c r="J64" s="86" t="s">
         <v>10</v>
       </c>
-      <c r="K61" s="87" t="s">
+      <c r="K64" s="86" t="s">
         <v>11</v>
       </c>
-      <c r="L61" s="87" t="s">
+      <c r="L64" s="86" t="s">
         <v>12</v>
       </c>
-      <c r="M61" s="87" t="s">
+      <c r="M64" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="N61" s="87" t="s">
+      <c r="N64" s="86" t="s">
         <v>14</v>
       </c>
-      <c r="O61" s="87" t="s">
+      <c r="O64" s="86" t="s">
         <v>41</v>
       </c>
-      <c r="P61" s="87" t="s">
+      <c r="P64" s="86" t="s">
         <v>15</v>
       </c>
-      <c r="Q61" s="87" t="s">
+      <c r="Q64" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="R61" s="87" t="s">
+      <c r="R64" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="S61" s="87" t="s">
+      <c r="S64" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="T61" s="87" t="s">
+      <c r="T64" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="U61" s="87" t="s">
+      <c r="U64" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="V61" s="87" t="s">
+      <c r="V64" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="W61" s="93" t="s">
+      <c r="W64" s="92" t="s">
         <v>42</v>
       </c>
-      <c r="X61" s="93" t="s">
+      <c r="X64" s="92" t="s">
         <v>43</v>
       </c>
-      <c r="Y61" s="93" t="s">
+      <c r="Y64" s="92" t="s">
         <v>44</v>
       </c>
-      <c r="Z61" s="93" t="s">
+      <c r="Z64" s="92" t="s">
         <v>45</v>
       </c>
-      <c r="AA61" s="93" t="s">
+      <c r="AA64" s="92" t="s">
         <v>46</v>
       </c>
-      <c r="AB61" s="87" t="s">
+      <c r="AB64" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="AC61" s="87" t="s">
+      <c r="AC64" s="86" t="s">
         <v>25</v>
       </c>
-      <c r="AD61" s="87" t="s">
+      <c r="AD64" s="86" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:31" ht="15" customHeight="1">
-      <c r="C62" s="94"/>
-      <c r="D62" s="95"/>
-      <c r="E62" s="96"/>
-      <c r="F62" s="97"/>
-      <c r="G62" s="97"/>
-      <c r="H62" s="98"/>
-      <c r="I62" s="99"/>
-      <c r="J62" s="99"/>
-      <c r="K62" s="99"/>
-      <c r="L62" s="100"/>
-      <c r="M62" s="100"/>
-      <c r="N62" s="100"/>
-      <c r="O62" s="101"/>
-      <c r="P62" s="100"/>
-      <c r="Q62" s="102"/>
-      <c r="R62" s="102"/>
-      <c r="S62" s="102"/>
-      <c r="T62" s="102"/>
-      <c r="U62" s="102"/>
-      <c r="V62" s="102"/>
-      <c r="W62" s="102"/>
-      <c r="X62" s="102"/>
-      <c r="Y62" s="102"/>
-      <c r="Z62" s="102"/>
-      <c r="AA62" s="102"/>
-      <c r="AB62" s="102"/>
-      <c r="AC62" s="102"/>
-      <c r="AD62" s="102"/>
+    <row r="65" spans="3:30" ht="15" customHeight="1">
+      <c r="C65" s="93"/>
+      <c r="D65" s="94"/>
+      <c r="E65" s="95"/>
+      <c r="F65" s="96"/>
+      <c r="G65" s="96"/>
+      <c r="H65" s="97"/>
+      <c r="I65" s="98"/>
+      <c r="J65" s="98"/>
+      <c r="K65" s="98"/>
+      <c r="L65" s="99"/>
+      <c r="M65" s="99"/>
+      <c r="N65" s="99"/>
+      <c r="O65" s="100"/>
+      <c r="P65" s="99"/>
+      <c r="Q65" s="101"/>
+      <c r="R65" s="101"/>
+      <c r="S65" s="101"/>
+      <c r="T65" s="101"/>
+      <c r="U65" s="101"/>
+      <c r="V65" s="101"/>
+      <c r="W65" s="101"/>
+      <c r="X65" s="101"/>
+      <c r="Y65" s="101"/>
+      <c r="Z65" s="101"/>
+      <c r="AA65" s="101"/>
+      <c r="AB65" s="101"/>
+      <c r="AC65" s="101"/>
+      <c r="AD65" s="101"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C39:D39"/>
     <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C36:D36"/>
   </mergeCells>
-  <conditionalFormatting sqref="I62:K62">
+  <conditionalFormatting sqref="I65:K65">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5564,7 +5605,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K55">
+  <conditionalFormatting sqref="K58">
     <cfRule type="cellIs" dxfId="82" priority="1" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
@@ -5572,7 +5613,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I55">
+  <conditionalFormatting sqref="I58">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5582,22 +5623,22 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F62">
+  <conditionalFormatting sqref="F65">
     <cfRule type="cellIs" dxfId="80" priority="10" operator="equal">
       <formula>"Definition"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G62">
+  <conditionalFormatting sqref="G65">
     <cfRule type="cellIs" dxfId="79" priority="9" operator="equal">
       <formula>"Note"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E55">
+  <conditionalFormatting sqref="E58">
     <cfRule type="cellIs" dxfId="78" priority="8" operator="equal">
       <formula>"Dataset Description"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F12:F14">
+  <conditionalFormatting sqref="F15:F17">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5607,17 +5648,17 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C62">
+  <conditionalFormatting sqref="C65">
     <cfRule type="cellIs" dxfId="77" priority="4" operator="equal">
       <formula>"Link"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C55">
+  <conditionalFormatting sqref="C58">
     <cfRule type="cellIs" dxfId="76" priority="3" operator="equal">
       <formula>"Link"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J55">
+  <conditionalFormatting sqref="J58">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5628,16 +5669,17 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="D59" location="'Country Stats'!A1" display="Country Stats" xr:uid="{37F97D7D-6476-49BF-9118-0DA3787A2751}"/>
+    <hyperlink ref="D62" location="'Country Stats'!A1" display="Country Stats" xr:uid="{37F97D7D-6476-49BF-9118-0DA3787A2751}"/>
+    <hyperlink ref="D10" r:id="rId1" xr:uid="{72FE398A-55A6-46EF-88FD-8804913A2E2A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
   <tableParts count="5">
-    <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
     <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5676,18 +5718,18 @@
       <c r="G2" s="76"/>
       <c r="H2" s="76"/>
     </row>
-    <row r="3" spans="1:8" ht="14.45" customHeight="1">
-      <c r="B3" s="84" t="str">
+    <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="B3" s="119" t="str">
         <f ca="1">HYPERLINK("#" &amp; CELL("address", _xlfn.XLOOKUP(Name,tbl_DfOverview[Dataframe],tbl_DfOverview[_],tbl_DfOverview[[#Headers],[_]])), "Overview ↩")</f>
         <v>Overview ↩</v>
       </c>
-      <c r="C3" s="84"/>
+      <c r="C3" s="83"/>
     </row>
     <row r="4" spans="1:8" ht="4.9000000000000004" customHeight="1">
       <c r="B4" s="69"/>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1">
-      <c r="B5" s="109" t="e" vm="1">
+      <c r="B5" s="108" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="C5" s="78" t="s">
@@ -5698,14 +5740,14 @@
     <row r="6" spans="1:8" ht="10.15" customHeight="1"/>
     <row r="7" spans="1:8">
       <c r="A7" s="67"/>
-      <c r="B7" s="86" t="s">
+      <c r="B7" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="10.15" customHeight="1">
+    <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="67"/>
     </row>
     <row r="9" spans="1:8" ht="49.9" hidden="1" customHeight="1" outlineLevel="1">
@@ -5801,14 +5843,14 @@
     <row r="22" spans="1:6" ht="10.15" customHeight="1"/>
     <row r="23" spans="1:6" outlineLevel="1">
       <c r="A23" s="67"/>
-      <c r="B23" s="86" t="s">
+      <c r="B23" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="24" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A24" s="67"/>
     </row>
     <row r="25" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
@@ -5890,14 +5932,14 @@
     <row r="35" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
     <row r="36" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A36" s="67"/>
-      <c r="B36" s="86" t="s">
+      <c r="B36" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="37" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A37" s="67"/>
     </row>
     <row r="38" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
@@ -5952,14 +5994,14 @@
     <row r="45" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
     <row r="46" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A46" s="67"/>
-      <c r="B46" s="86" t="s">
+      <c r="B46" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="47" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A47" s="67"/>
     </row>
     <row r="48" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
@@ -6045,14 +6087,14 @@
     <row r="57" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
     <row r="58" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A58" s="67"/>
-      <c r="B58" s="86" t="s">
+      <c r="B58" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="59" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A59" s="67"/>
     </row>
     <row r="60" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
@@ -6177,14 +6219,14 @@
     <row r="68" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
     <row r="69" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A69" s="67"/>
-      <c r="B69" s="86" t="s">
+      <c r="B69" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="70" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A70" s="67"/>
     </row>
     <row r="71" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">

</xml_diff>

<commit_message>
Added theme setting and vba toggling to cli More readme polish Minor test updates Added documentation link to template
</commit_message>
<xml_diff>
--- a/src/xleda/xleda_template.xlsx
+++ b/src/xleda/xleda_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\.xleda\src\xleda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8FA3A98-AC7F-49B5-BE3A-E5583C25AD62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CAF48AD-2D47-46BA-9472-C55952E2D062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="735" firstSheet="1" activeTab="1" xr2:uid="{040F3586-419E-4585-8ACE-6588AD7C95BD}"/>
   </bookViews>
@@ -18,21 +18,21 @@
     <sheet name="Field Analysis" sheetId="25" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="Back">Overview!$D$54</definedName>
+    <definedName name="Back">Overview!$D$57</definedName>
     <definedName name="Compiled_Lists" localSheetId="2">'Field Analysis'!$C$71:$C$80</definedName>
     <definedName name="Composition" localSheetId="2">'Field Analysis'!$C$25:$C$35</definedName>
     <definedName name="CompositionTable" localSheetId="2">'Field Analysis'!$D$34</definedName>
     <definedName name="DarkHeader" localSheetId="2">'Field Analysis'!$D$81</definedName>
     <definedName name="Data_Description" localSheetId="2">'Field Analysis'!$C$9:$C$20</definedName>
-    <definedName name="Dataframes">Overview!$C$54:$C$57</definedName>
-    <definedName name="Debug" localSheetId="1">Overview!$D$9:$E$51</definedName>
+    <definedName name="Dataframes">Overview!$C$57:$C$60</definedName>
+    <definedName name="Debug" localSheetId="1">Overview!$D$9:$E$54</definedName>
     <definedName name="DebugToggle" localSheetId="1">Overview!$B$6</definedName>
     <definedName name="Definitions" localSheetId="2">'Field Analysis'!$D$17:$F$17</definedName>
     <definedName name="Description" localSheetId="2">'Field Analysis'!$D$9</definedName>
     <definedName name="Dimensions" localSheetId="2">'Field Analysis'!$D$11</definedName>
     <definedName name="Field_Analysis" localSheetId="2">'Field Analysis'!$D$22:$D$80</definedName>
     <definedName name="Field_Lists" localSheetId="2">'Field Analysis'!$C$60:$C$68</definedName>
-    <definedName name="Field_Overview">Overview!$E$61:$E$62</definedName>
+    <definedName name="Field_Overview">Overview!$E$64:$E$65</definedName>
     <definedName name="FieldList1" localSheetId="2">'Field Analysis'!$D$60:$F$60</definedName>
     <definedName name="FieldList2" localSheetId="2">'Field Analysis'!$D$61:$F$61</definedName>
     <definedName name="FieldList3" localSheetId="2">'Field Analysis'!$D$62:$F$62</definedName>
@@ -43,7 +43,7 @@
     <definedName name="FieldList8" localSheetId="2">'Field Analysis'!$D$67:$F$67</definedName>
     <definedName name="FieldLists" localSheetId="2">'Field Analysis'!$C$60:$F$67</definedName>
     <definedName name="FieldRange" localSheetId="2">'Field Analysis'!$D$81:$F$81</definedName>
-    <definedName name="Fields">Overview!$C$61:$C$62</definedName>
+    <definedName name="Fields">Overview!$C$64:$C$65</definedName>
     <definedName name="FormatRange" localSheetId="2">'Field Analysis'!$F:$F</definedName>
     <definedName name="Headers" localSheetId="2">'Field Analysis'!$D$21:$F$21</definedName>
     <definedName name="Headers_Start" localSheetId="2">'Field Analysis'!$D$21</definedName>
@@ -58,7 +58,7 @@
     <definedName name="SinglePlot" localSheetId="0">SinglePlot!$C$10</definedName>
     <definedName name="Summary_Stats" localSheetId="2">'Field Analysis'!$C$38:$C$45</definedName>
     <definedName name="Theme" localSheetId="2">'Field Analysis'!$B$21:$F$21</definedName>
-    <definedName name="Theme" localSheetId="1">Overview!$E$61:$AD$61</definedName>
+    <definedName name="Theme" localSheetId="1">Overview!$E$64:$AD$64</definedName>
     <definedName name="Theme" localSheetId="0">SinglePlot!$B$8:$P$8</definedName>
     <definedName name="Toggles" localSheetId="2">'Field Analysis'!$B$7,'Field Analysis'!$B$23,'Field Analysis'!$B$36,'Field Analysis'!$B$46,'Field Analysis'!$B$58,'Field Analysis'!$B$69</definedName>
     <definedName name="TopToggle" localSheetId="2">'Field Analysis'!$B$5</definedName>
@@ -125,7 +125,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="108">
   <si>
     <t>Warning</t>
   </si>
@@ -443,6 +443,12 @@
   </si>
   <si>
     <t>data argument</t>
+  </si>
+  <si>
+    <t>xleda Documentation:</t>
+  </si>
+  <si>
+    <t>https://github.com/InfoDesigner/xleda/</t>
   </si>
 </sst>
 </file>
@@ -705,13 +711,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="4"/>
-      <color theme="1" tint="0.39997558519241921"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <i/>
       <sz val="6"/>
@@ -723,6 +722,15 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1" tint="0.39997558519241921"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="8"/>
       <color theme="1" tint="0.39997558519241921"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1063,7 +1071,7 @@
     </xf>
     <xf numFmtId="9" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" textRotation="180"/>
@@ -1287,10 +1295,7 @@
     <xf numFmtId="3" fontId="10" fillId="8" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -1373,13 +1378,13 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="35" fillId="5" borderId="16" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="34" fillId="5" borderId="16" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="35" fillId="5" borderId="19" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="3" fontId="34" fillId="5" borderId="19" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="35" fillId="5" borderId="17" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="3" fontId="34" fillId="5" borderId="17" xfId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="10" fillId="2" borderId="18" xfId="7" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1387,6 +1392,13 @@
     </xf>
     <xf numFmtId="3" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="3" applyFont="1" applyBorder="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="32" fillId="2" borderId="0" xfId="7" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -4353,7 +4365,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E2133564-163D-4CB0-A97C-9358270F5F9C}" name="tbl_debug_section" displayName="tbl_debug_section" ref="D11:F14" totalsRowShown="0" headerRowDxfId="75" dataDxfId="73" headerRowBorderDxfId="74" tableBorderDxfId="72" totalsRowBorderDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E2133564-163D-4CB0-A97C-9358270F5F9C}" name="tbl_debug_section" displayName="tbl_debug_section" ref="D14:F17" totalsRowShown="0" headerRowDxfId="75" dataDxfId="73" headerRowBorderDxfId="74" tableBorderDxfId="72" totalsRowBorderDxfId="71">
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5EB43B6F-4FF7-4D4C-8202-BD94842B8017}" name="Production Section" dataDxfId="70" dataCellStyle="DarkHeader"/>
     <tableColumn id="2" xr3:uid="{71F0A434-8F03-4CF9-987C-D6F88D936E0A}" name="Production Time in Seconds" dataDxfId="69"/>
@@ -4364,7 +4376,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FABCC19D-29F4-4A1C-9C2C-61132A93E32D}" name="tbl_debug_environment" displayName="tbl_debug_environment" ref="D19:E33" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FABCC19D-29F4-4A1C-9C2C-61132A93E32D}" name="tbl_debug_environment" displayName="tbl_debug_environment" ref="D22:E36" totalsRowShown="0" headerRowDxfId="67" dataDxfId="65" headerRowBorderDxfId="66" tableBorderDxfId="64">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{6A891059-3C09-438F-9AB9-42F8BA5B3379}" name="Environment Variable" dataDxfId="63" dataCellStyle="DarkHeader"/>
     <tableColumn id="2" xr3:uid="{D9E0C91D-D549-4194-8575-1343B51883A7}" name="Value" dataDxfId="62"/>
@@ -4374,7 +4386,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{88D10CD5-62A0-484D-A455-84E38CB47746}" name="tbl_debug_config" displayName="tbl_debug_config" ref="D38:E50" totalsRowShown="0" headerRowDxfId="61" headerRowBorderDxfId="60" tableBorderDxfId="59" totalsRowBorderDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{88D10CD5-62A0-484D-A455-84E38CB47746}" name="tbl_debug_config" displayName="tbl_debug_config" ref="D41:E53" totalsRowShown="0" headerRowDxfId="61" headerRowBorderDxfId="60" tableBorderDxfId="59" totalsRowBorderDxfId="58">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{BAFB02A5-6AA3-46EF-A3FA-1FC44F32BBF4}" name="Input Argument" dataDxfId="57" dataCellStyle="DarkHeader"/>
     <tableColumn id="2" xr3:uid="{402A365F-6164-4790-9B23-3CC27E2F5642}" name="Value" dataDxfId="56" dataCellStyle="DarkHeader"/>
@@ -4384,7 +4396,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AFE650AA-A988-4967-9BF1-5CBBD5AE48A6}" name="tbl_FieldOverview" displayName="tbl_FieldOverview" ref="C61:AD62" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AFE650AA-A988-4967-9BF1-5CBBD5AE48A6}" name="tbl_FieldOverview" displayName="tbl_FieldOverview" ref="C64:AD65" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54">
   <tableColumns count="28">
     <tableColumn id="1" xr3:uid="{BFB84B7E-8B25-47B3-90FE-AC7BFBAF30EB}" name="_" dataDxfId="52" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{50D3F477-2874-418A-8431-FEC88B724332}" name="Dataframe" dataDxfId="51"/>
@@ -4420,7 +4432,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B62C177-35BB-4328-A5E9-CE2D42C175A6}" name="tbl_DfOverview" displayName="tbl_DfOverview" ref="C54:K55" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0B62C177-35BB-4328-A5E9-CE2D42C175A6}" name="tbl_DfOverview" displayName="tbl_DfOverview" ref="C57:K58" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{95AE6ED1-2225-487F-9D3B-3E94D426571D}" name="_" dataDxfId="21" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{19718F20-2450-421A-9215-32A414225B3E}" name="Dataframe" dataDxfId="20" dataCellStyle="Hyperlink"/>
@@ -4799,17 +4811,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="4.9000000000000004" customHeight="1"/>
-    <row r="2" spans="2:16" ht="14.45" customHeight="1">
-      <c r="B2" s="84" t="s">
+    <row r="2" spans="2:16" ht="20.100000000000001" customHeight="1">
+      <c r="B2" s="119" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="84"/>
+      <c r="D2" s="83"/>
     </row>
     <row r="3" spans="2:16" ht="10.15" customHeight="1">
       <c r="B3" s="77"/>
     </row>
     <row r="4" spans="2:16" ht="30" customHeight="1">
-      <c r="B4" s="109" t="e" vm="1">
+      <c r="B4" s="108" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="C4" s="53" t="s">
@@ -4879,7 +4891,7 @@
     <tabColor theme="4"/>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:AE62"/>
+  <dimension ref="A1:AE65"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="1.7109375" customWidth="1"/>
@@ -4893,7 +4905,7 @@
     <col min="21" max="30" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="85" customFormat="1" ht="4.9000000000000004" customHeight="1">
+    <row r="1" spans="1:28" s="84" customFormat="1" ht="4.9000000000000004" customHeight="1">
       <c r="H1"/>
       <c r="I1"/>
       <c r="J1"/>
@@ -4901,14 +4913,14 @@
     <row r="2" spans="1:28" ht="14.45" customHeight="1">
       <c r="A2" s="71"/>
     </row>
-    <row r="3" spans="1:28" s="85" customFormat="1" ht="10.15" customHeight="1">
+    <row r="3" spans="1:28" s="84" customFormat="1" ht="10.15" customHeight="1">
       <c r="A3" s="71"/>
       <c r="H3"/>
       <c r="I3"/>
       <c r="J3"/>
     </row>
     <row r="4" spans="1:28" ht="30" customHeight="1">
-      <c r="B4" s="110" t="e" vm="1">
+      <c r="B4" s="109" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="C4" s="53" t="s">
@@ -4917,15 +4929,15 @@
       <c r="D4" s="74"/>
       <c r="AB4" s="4"/>
     </row>
-    <row r="5" spans="1:28" ht="10.15" customHeight="1">
+    <row r="5" spans="1:28" ht="20.100000000000001" customHeight="1">
       <c r="C5" s="53"/>
       <c r="AB5" s="4"/>
     </row>
     <row r="6" spans="1:28" ht="15" customHeight="1">
-      <c r="B6" s="83" t="s">
+      <c r="B6" s="118" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="84" t="s">
+      <c r="C6" s="119" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="51"/>
@@ -4942,236 +4954,222 @@
       <c r="G7" s="43"/>
       <c r="K7" s="43"/>
     </row>
-    <row r="8" spans="1:28" ht="15" customHeight="1">
+    <row r="8" spans="1:28" ht="20.100000000000001" customHeight="1">
       <c r="C8" s="43"/>
       <c r="D8" s="43"/>
       <c r="E8" s="43"/>
       <c r="F8" s="43"/>
-      <c r="G8" s="111"/>
+      <c r="G8" s="110"/>
       <c r="K8" s="43"/>
     </row>
-    <row r="9" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B9" s="1"/>
-      <c r="C9" s="118" t="s">
+    <row r="9" spans="1:28" s="84" customFormat="1" ht="30" hidden="1" customHeight="1">
+      <c r="C9" s="120" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="120"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="117"/>
+      <c r="K9" s="43"/>
+    </row>
+    <row r="10" spans="1:28" s="84" customFormat="1" ht="15" hidden="1" customHeight="1">
+      <c r="C10" s="43"/>
+      <c r="D10" s="82" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="117"/>
+      <c r="K10" s="43"/>
+    </row>
+    <row r="11" spans="1:28" s="84" customFormat="1" ht="15" hidden="1" customHeight="1">
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="117"/>
+      <c r="K11" s="43"/>
+    </row>
+    <row r="12" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B12" s="1"/>
+      <c r="C12" s="120" t="s">
         <v>97</v>
       </c>
-      <c r="D9" s="118"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="K9" s="43"/>
-    </row>
-    <row r="10" spans="1:28" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-    </row>
-    <row r="11" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B11" s="41"/>
-      <c r="D11" s="113" t="s">
+      <c r="D12" s="120"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="K12" s="43"/>
+    </row>
+    <row r="13" spans="1:28" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
+    </row>
+    <row r="14" spans="1:28" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B14" s="41"/>
+      <c r="D14" s="112" t="s">
         <v>56</v>
       </c>
-      <c r="E11" s="115" t="s">
+      <c r="E14" s="114" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="114" t="s">
+      <c r="F14" s="113" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D12" s="116" t="s">
+    <row r="15" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D15" s="115" t="s">
         <v>101</v>
       </c>
-      <c r="E12" s="50"/>
-      <c r="F12" s="49"/>
-    </row>
-    <row r="13" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D13" s="116" t="s">
+      <c r="E15" s="50"/>
+      <c r="F15" s="49"/>
+    </row>
+    <row r="16" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D16" s="115" t="s">
         <v>102</v>
       </c>
-      <c r="E13" s="50"/>
-      <c r="F13" s="49"/>
-    </row>
-    <row r="14" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D14" s="116" t="s">
+      <c r="E16" s="50"/>
+      <c r="F16" s="49"/>
+    </row>
+    <row r="17" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D17" s="115" t="s">
         <v>59</v>
       </c>
-      <c r="E14" s="50"/>
-      <c r="F14" s="49"/>
-    </row>
-    <row r="15" spans="1:28" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-    </row>
-    <row r="16" spans="1:28" ht="10.15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="L16" s="38"/>
-    </row>
-    <row r="17" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C17" s="118" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="118"/>
-      <c r="E17" s="80"/>
-      <c r="L17" s="38"/>
-    </row>
-    <row r="18" spans="2:12" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="E17" s="50"/>
+      <c r="F17" s="49"/>
+    </row>
+    <row r="18" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C18" s="43"/>
       <c r="D18" s="43"/>
       <c r="E18" s="43"/>
     </row>
-    <row r="19" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D19" s="113" t="s">
+    <row r="19" spans="2:12" ht="10.15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="L19" s="38"/>
+    </row>
+    <row r="20" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C20" s="120" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="120"/>
+      <c r="E20" s="80"/>
+      <c r="L20" s="38"/>
+    </row>
+    <row r="21" spans="2:12" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+    </row>
+    <row r="22" spans="2:12" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D22" s="112" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="114" t="s">
+      <c r="E22" s="113" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="20" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D20" s="44" t="s">
-        <v>62</v>
-      </c>
-      <c r="E20" s="56"/>
-    </row>
-    <row r="21" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D21" s="44" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" s="56"/>
-    </row>
-    <row r="22" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D22" s="44" t="s">
-        <v>64</v>
-      </c>
-      <c r="E22" s="56"/>
     </row>
     <row r="23" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D23" s="44" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E23" s="56"/>
     </row>
     <row r="24" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D24" s="44" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E24" s="56"/>
     </row>
     <row r="25" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D25" s="44" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E25" s="56"/>
     </row>
     <row r="26" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D26" s="44" t="s">
-        <v>69</v>
-      </c>
-      <c r="E26" s="57"/>
+        <v>66</v>
+      </c>
+      <c r="E26" s="56"/>
     </row>
     <row r="27" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D27" s="44" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E27" s="56"/>
     </row>
     <row r="28" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B28" s="39"/>
       <c r="D28" s="44" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E28" s="56"/>
     </row>
     <row r="29" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D29" s="44" t="s">
-        <v>72</v>
-      </c>
-      <c r="E29" s="56"/>
+        <v>69</v>
+      </c>
+      <c r="E29" s="57"/>
     </row>
     <row r="30" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D30" s="44" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E30" s="56"/>
     </row>
     <row r="31" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B31" s="39"/>
       <c r="D31" s="44" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E31" s="56"/>
-      <c r="I31" s="81"/>
-      <c r="J31" s="82"/>
-      <c r="K31" s="43"/>
     </row>
     <row r="32" spans="2:12" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D32" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" s="56"/>
+    </row>
+    <row r="33" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D33" s="44" t="s">
+        <v>73</v>
+      </c>
+      <c r="E33" s="56"/>
+    </row>
+    <row r="34" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D34" s="44" t="s">
+        <v>74</v>
+      </c>
+      <c r="E34" s="56"/>
+      <c r="I34" s="81"/>
+      <c r="J34" s="82"/>
+      <c r="K34" s="43"/>
+    </row>
+    <row r="35" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D35" s="44" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="56"/>
-      <c r="K32" s="43"/>
-    </row>
-    <row r="33" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B33" s="40"/>
-      <c r="C33" s="45"/>
-      <c r="D33" s="44" t="s">
+      <c r="E35" s="56"/>
+      <c r="K35" s="43"/>
+    </row>
+    <row r="36" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B36" s="40"/>
+      <c r="C36" s="45"/>
+      <c r="D36" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="E33" s="56"/>
-      <c r="K33" s="43"/>
-    </row>
-    <row r="34" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="B34" s="40"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="81"/>
-      <c r="E34" s="56"/>
-      <c r="K34" s="43"/>
-    </row>
-    <row r="35" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D35" s="47"/>
-      <c r="E35" s="46"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="43"/>
-      <c r="I35" s="43"/>
-      <c r="J35" s="43"/>
-      <c r="K35" s="43"/>
-      <c r="W35" s="42"/>
-      <c r="Y35" s="38"/>
-    </row>
-    <row r="36" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="C36" s="118" t="s">
-        <v>53</v>
-      </c>
-      <c r="D36" s="118"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="43"/>
-      <c r="I36" s="43"/>
-      <c r="J36" s="43"/>
+      <c r="E36" s="56"/>
       <c r="K36" s="43"/>
-      <c r="W36" s="42"/>
-      <c r="Y36" s="38"/>
-    </row>
-    <row r="37" spans="2:25" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="43"/>
-      <c r="I37" s="43"/>
-      <c r="J37" s="43"/>
+    </row>
+    <row r="37" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="B37" s="40"/>
+      <c r="C37" s="45"/>
+      <c r="D37" s="81"/>
+      <c r="E37" s="56"/>
       <c r="K37" s="43"/>
-      <c r="W37" s="42"/>
-      <c r="Y37" s="38"/>
-    </row>
-    <row r="38" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D38" s="113" t="s">
-        <v>60</v>
-      </c>
-      <c r="E38" s="114" t="s">
-        <v>55</v>
-      </c>
+    </row>
+    <row r="38" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D38" s="47"/>
+      <c r="E38" s="46"/>
       <c r="F38" s="43"/>
       <c r="G38" s="43"/>
       <c r="H38" s="43"/>
@@ -5181,11 +5179,11 @@
       <c r="W38" s="42"/>
       <c r="Y38" s="38"/>
     </row>
-    <row r="39" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D39" s="48" t="s">
-        <v>103</v>
-      </c>
-      <c r="E39" s="54"/>
+    <row r="39" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="C39" s="120" t="s">
+        <v>53</v>
+      </c>
+      <c r="D39" s="120"/>
       <c r="F39" s="43"/>
       <c r="G39" s="43"/>
       <c r="H39" s="43"/>
@@ -5195,11 +5193,9 @@
       <c r="W39" s="42"/>
       <c r="Y39" s="38"/>
     </row>
-    <row r="40" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D40" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="E40" s="55"/>
+    <row r="40" spans="2:25" ht="4.9000000000000004" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
       <c r="F40" s="43"/>
       <c r="G40" s="43"/>
       <c r="H40" s="43"/>
@@ -5209,11 +5205,13 @@
       <c r="W40" s="42"/>
       <c r="Y40" s="38"/>
     </row>
-    <row r="41" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D41" s="64" t="s">
-        <v>105</v>
-      </c>
-      <c r="E41" s="55"/>
+    <row r="41" spans="2:25" ht="30" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D41" s="112" t="s">
+        <v>60</v>
+      </c>
+      <c r="E41" s="113" t="s">
+        <v>55</v>
+      </c>
       <c r="F41" s="43"/>
       <c r="G41" s="43"/>
       <c r="H41" s="43"/>
@@ -5224,10 +5222,10 @@
       <c r="Y41" s="38"/>
     </row>
     <row r="42" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D42" s="64" t="s">
-        <v>77</v>
-      </c>
-      <c r="E42" s="55"/>
+      <c r="D42" s="48" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" s="54"/>
       <c r="F42" s="43"/>
       <c r="G42" s="43"/>
       <c r="H42" s="43"/>
@@ -5238,8 +5236,8 @@
       <c r="Y42" s="38"/>
     </row>
     <row r="43" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D43" s="64" t="s">
-        <v>78</v>
+      <c r="D43" s="44" t="s">
+        <v>104</v>
       </c>
       <c r="E43" s="55"/>
       <c r="F43" s="43"/>
@@ -5253,7 +5251,7 @@
     </row>
     <row r="44" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D44" s="64" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="E44" s="55"/>
       <c r="F44" s="43"/>
@@ -5267,7 +5265,7 @@
     </row>
     <row r="45" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D45" s="64" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E45" s="55"/>
       <c r="F45" s="43"/>
@@ -5281,7 +5279,7 @@
     </row>
     <row r="46" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D46" s="64" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E46" s="55"/>
       <c r="F46" s="43"/>
@@ -5295,7 +5293,7 @@
     </row>
     <row r="47" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D47" s="64" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E47" s="55"/>
       <c r="F47" s="43"/>
@@ -5308,10 +5306,10 @@
       <c r="Y47" s="38"/>
     </row>
     <row r="48" spans="2:25" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D48" s="65" t="s">
-        <v>83</v>
-      </c>
-      <c r="E48" s="66"/>
+      <c r="D48" s="64" t="s">
+        <v>80</v>
+      </c>
+      <c r="E48" s="55"/>
       <c r="F48" s="43"/>
       <c r="G48" s="43"/>
       <c r="H48" s="43"/>
@@ -5323,7 +5321,7 @@
     </row>
     <row r="49" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
       <c r="D49" s="64" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E49" s="55"/>
       <c r="F49" s="43"/>
@@ -5336,10 +5334,10 @@
       <c r="Y49" s="38"/>
     </row>
     <row r="50" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D50" s="65" t="s">
-        <v>65</v>
-      </c>
-      <c r="E50" s="66"/>
+      <c r="D50" s="64" t="s">
+        <v>82</v>
+      </c>
+      <c r="E50" s="55"/>
       <c r="F50" s="43"/>
       <c r="G50" s="43"/>
       <c r="H50" s="43"/>
@@ -5350,8 +5348,10 @@
       <c r="Y50" s="38"/>
     </row>
     <row r="51" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
-      <c r="D51" s="47"/>
-      <c r="E51" s="46"/>
+      <c r="D51" s="65" t="s">
+        <v>83</v>
+      </c>
+      <c r="E51" s="66"/>
       <c r="F51" s="43"/>
       <c r="G51" s="43"/>
       <c r="H51" s="43"/>
@@ -5361,200 +5361,241 @@
       <c r="W51" s="42"/>
       <c r="Y51" s="38"/>
     </row>
-    <row r="52" spans="1:31" ht="15" customHeight="1" collapsed="1">
-      <c r="A52" s="6"/>
-      <c r="B52" s="68" t="s">
+    <row r="52" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D52" s="64" t="s">
+        <v>84</v>
+      </c>
+      <c r="E52" s="55"/>
+      <c r="F52" s="43"/>
+      <c r="G52" s="43"/>
+      <c r="H52" s="43"/>
+      <c r="I52" s="43"/>
+      <c r="J52" s="43"/>
+      <c r="K52" s="43"/>
+      <c r="W52" s="42"/>
+      <c r="Y52" s="38"/>
+    </row>
+    <row r="53" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D53" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="E53" s="66"/>
+      <c r="F53" s="43"/>
+      <c r="G53" s="43"/>
+      <c r="H53" s="43"/>
+      <c r="I53" s="43"/>
+      <c r="J53" s="43"/>
+      <c r="K53" s="43"/>
+      <c r="W53" s="42"/>
+      <c r="Y53" s="38"/>
+    </row>
+    <row r="54" spans="1:31" ht="15" hidden="1" customHeight="1" outlineLevel="1">
+      <c r="D54" s="47"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="43"/>
+      <c r="G54" s="43"/>
+      <c r="H54" s="43"/>
+      <c r="I54" s="43"/>
+      <c r="J54" s="43"/>
+      <c r="K54" s="43"/>
+      <c r="W54" s="42"/>
+      <c r="Y54" s="38"/>
+    </row>
+    <row r="55" spans="1:31" ht="15" customHeight="1" collapsed="1">
+      <c r="A55" s="6"/>
+      <c r="B55" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="C52" s="112" t="s">
+      <c r="C55" s="111" t="s">
         <v>87</v>
       </c>
-      <c r="AB52" s="4"/>
-    </row>
-    <row r="53" spans="1:31" ht="15" customHeight="1">
-      <c r="C53" s="53"/>
-      <c r="AB53" s="4"/>
-    </row>
-    <row r="54" spans="1:31" ht="30" customHeight="1">
-      <c r="C54" s="88" t="s">
+      <c r="AB55" s="4"/>
+    </row>
+    <row r="56" spans="1:31" ht="20.100000000000001" customHeight="1">
+      <c r="C56" s="53"/>
+      <c r="AB56" s="4"/>
+    </row>
+    <row r="57" spans="1:31" ht="30" customHeight="1">
+      <c r="C57" s="87" t="s">
         <v>91</v>
       </c>
-      <c r="D54" s="89" t="s">
+      <c r="D57" s="88" t="s">
         <v>86</v>
       </c>
-      <c r="E54" s="90" t="s">
+      <c r="E57" s="89" t="s">
         <v>100</v>
       </c>
-      <c r="F54" s="87" t="s">
+      <c r="F57" s="86" t="s">
         <v>89</v>
       </c>
-      <c r="G54" s="91" t="s">
+      <c r="G57" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="H54" s="91" t="s">
+      <c r="H57" s="90" t="s">
         <v>48</v>
       </c>
-      <c r="I54" s="91" t="s">
+      <c r="I57" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="J54" s="91" t="s">
+      <c r="J57" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="K54" s="87" t="s">
+      <c r="K57" s="86" t="s">
         <v>98</v>
       </c>
-      <c r="AE54" s="4"/>
-    </row>
-    <row r="55" spans="1:31" ht="15" customHeight="1">
-      <c r="C55" s="94"/>
-      <c r="D55" s="103"/>
-      <c r="E55" s="104"/>
-      <c r="F55" s="117"/>
-      <c r="G55" s="105"/>
-      <c r="H55" s="106"/>
-      <c r="I55" s="107"/>
-      <c r="J55" s="99"/>
-      <c r="K55" s="108"/>
-      <c r="AE55" s="4"/>
-    </row>
-    <row r="57" spans="1:31" ht="15" customHeight="1">
-      <c r="AB57" s="4"/>
+      <c r="AE57" s="4"/>
     </row>
     <row r="58" spans="1:31" ht="15" customHeight="1">
-      <c r="B58" s="68" t="s">
+      <c r="C58" s="93"/>
+      <c r="D58" s="102"/>
+      <c r="E58" s="103"/>
+      <c r="F58" s="116"/>
+      <c r="G58" s="104"/>
+      <c r="H58" s="105"/>
+      <c r="I58" s="106"/>
+      <c r="J58" s="98"/>
+      <c r="K58" s="107"/>
+      <c r="AE58" s="4"/>
+    </row>
+    <row r="60" spans="1:31" ht="15" customHeight="1">
+      <c r="AB60" s="4"/>
+    </row>
+    <row r="61" spans="1:31" ht="15" customHeight="1">
+      <c r="B61" s="68" t="s">
         <v>61</v>
       </c>
-      <c r="C58" s="112" t="s">
+      <c r="C61" s="111" t="s">
         <v>88</v>
       </c>
-      <c r="D58" s="85"/>
-      <c r="AB58" s="4"/>
-    </row>
-    <row r="59" spans="1:31" ht="10.15" customHeight="1"/>
-    <row r="60" spans="1:31" ht="10.15" customHeight="1"/>
-    <row r="61" spans="1:31" ht="30" customHeight="1">
-      <c r="C61" s="88" t="s">
+      <c r="D61" s="84"/>
+      <c r="AB61" s="4"/>
+    </row>
+    <row r="62" spans="1:31" ht="20.100000000000001" customHeight="1"/>
+    <row r="63" spans="1:31" ht="10.15" customHeight="1"/>
+    <row r="64" spans="1:31" ht="30" customHeight="1">
+      <c r="C64" s="87" t="s">
         <v>91</v>
       </c>
-      <c r="D61" s="92" t="s">
+      <c r="D64" s="91" t="s">
         <v>86</v>
       </c>
-      <c r="E61" s="92" t="s">
+      <c r="E64" s="91" t="s">
         <v>39</v>
       </c>
-      <c r="F61" s="92" t="s">
+      <c r="F64" s="91" t="s">
         <v>40</v>
       </c>
-      <c r="G61" s="92" t="s">
+      <c r="G64" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="H61" s="87" t="s">
+      <c r="H64" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="I61" s="87" t="s">
+      <c r="I64" s="86" t="s">
         <v>9</v>
       </c>
-      <c r="J61" s="87" t="s">
+      <c r="J64" s="86" t="s">
         <v>10</v>
       </c>
-      <c r="K61" s="87" t="s">
+      <c r="K64" s="86" t="s">
         <v>11</v>
       </c>
-      <c r="L61" s="87" t="s">
+      <c r="L64" s="86" t="s">
         <v>12</v>
       </c>
-      <c r="M61" s="87" t="s">
+      <c r="M64" s="86" t="s">
         <v>13</v>
       </c>
-      <c r="N61" s="87" t="s">
+      <c r="N64" s="86" t="s">
         <v>14</v>
       </c>
-      <c r="O61" s="87" t="s">
+      <c r="O64" s="86" t="s">
         <v>41</v>
       </c>
-      <c r="P61" s="87" t="s">
+      <c r="P64" s="86" t="s">
         <v>15</v>
       </c>
-      <c r="Q61" s="87" t="s">
+      <c r="Q64" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="R61" s="87" t="s">
+      <c r="R64" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="S61" s="87" t="s">
+      <c r="S64" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="T61" s="87" t="s">
+      <c r="T64" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="U61" s="87" t="s">
+      <c r="U64" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="V61" s="87" t="s">
+      <c r="V64" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="W61" s="93" t="s">
+      <c r="W64" s="92" t="s">
         <v>42</v>
       </c>
-      <c r="X61" s="93" t="s">
+      <c r="X64" s="92" t="s">
         <v>43</v>
       </c>
-      <c r="Y61" s="93" t="s">
+      <c r="Y64" s="92" t="s">
         <v>44</v>
       </c>
-      <c r="Z61" s="93" t="s">
+      <c r="Z64" s="92" t="s">
         <v>45</v>
       </c>
-      <c r="AA61" s="93" t="s">
+      <c r="AA64" s="92" t="s">
         <v>46</v>
       </c>
-      <c r="AB61" s="87" t="s">
+      <c r="AB64" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="AC61" s="87" t="s">
+      <c r="AC64" s="86" t="s">
         <v>25</v>
       </c>
-      <c r="AD61" s="87" t="s">
+      <c r="AD64" s="86" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="62" spans="1:31" ht="15" customHeight="1">
-      <c r="C62" s="94"/>
-      <c r="D62" s="95"/>
-      <c r="E62" s="96"/>
-      <c r="F62" s="97"/>
-      <c r="G62" s="97"/>
-      <c r="H62" s="98"/>
-      <c r="I62" s="99"/>
-      <c r="J62" s="99"/>
-      <c r="K62" s="99"/>
-      <c r="L62" s="100"/>
-      <c r="M62" s="100"/>
-      <c r="N62" s="100"/>
-      <c r="O62" s="101"/>
-      <c r="P62" s="100"/>
-      <c r="Q62" s="102"/>
-      <c r="R62" s="102"/>
-      <c r="S62" s="102"/>
-      <c r="T62" s="102"/>
-      <c r="U62" s="102"/>
-      <c r="V62" s="102"/>
-      <c r="W62" s="102"/>
-      <c r="X62" s="102"/>
-      <c r="Y62" s="102"/>
-      <c r="Z62" s="102"/>
-      <c r="AA62" s="102"/>
-      <c r="AB62" s="102"/>
-      <c r="AC62" s="102"/>
-      <c r="AD62" s="102"/>
+    <row r="65" spans="3:30" ht="15" customHeight="1">
+      <c r="C65" s="93"/>
+      <c r="D65" s="94"/>
+      <c r="E65" s="95"/>
+      <c r="F65" s="96"/>
+      <c r="G65" s="96"/>
+      <c r="H65" s="97"/>
+      <c r="I65" s="98"/>
+      <c r="J65" s="98"/>
+      <c r="K65" s="98"/>
+      <c r="L65" s="99"/>
+      <c r="M65" s="99"/>
+      <c r="N65" s="99"/>
+      <c r="O65" s="100"/>
+      <c r="P65" s="99"/>
+      <c r="Q65" s="101"/>
+      <c r="R65" s="101"/>
+      <c r="S65" s="101"/>
+      <c r="T65" s="101"/>
+      <c r="U65" s="101"/>
+      <c r="V65" s="101"/>
+      <c r="W65" s="101"/>
+      <c r="X65" s="101"/>
+      <c r="Y65" s="101"/>
+      <c r="Z65" s="101"/>
+      <c r="AA65" s="101"/>
+      <c r="AB65" s="101"/>
+      <c r="AC65" s="101"/>
+      <c r="AD65" s="101"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C39:D39"/>
     <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C36:D36"/>
   </mergeCells>
-  <conditionalFormatting sqref="I62:K62">
+  <conditionalFormatting sqref="I65:K65">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5564,7 +5605,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K55">
+  <conditionalFormatting sqref="K58">
     <cfRule type="cellIs" dxfId="82" priority="1" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
@@ -5572,7 +5613,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I55">
+  <conditionalFormatting sqref="I58">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5582,22 +5623,22 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F62">
+  <conditionalFormatting sqref="F65">
     <cfRule type="cellIs" dxfId="80" priority="10" operator="equal">
       <formula>"Definition"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G62">
+  <conditionalFormatting sqref="G65">
     <cfRule type="cellIs" dxfId="79" priority="9" operator="equal">
       <formula>"Note"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E55">
+  <conditionalFormatting sqref="E58">
     <cfRule type="cellIs" dxfId="78" priority="8" operator="equal">
       <formula>"Dataset Description"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F12:F14">
+  <conditionalFormatting sqref="F15:F17">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5607,17 +5648,17 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C62">
+  <conditionalFormatting sqref="C65">
     <cfRule type="cellIs" dxfId="77" priority="4" operator="equal">
       <formula>"Link"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C55">
+  <conditionalFormatting sqref="C58">
     <cfRule type="cellIs" dxfId="76" priority="3" operator="equal">
       <formula>"Link"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J55">
+  <conditionalFormatting sqref="J58">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5628,16 +5669,17 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="D59" location="'Country Stats'!A1" display="Country Stats" xr:uid="{37F97D7D-6476-49BF-9118-0DA3787A2751}"/>
+    <hyperlink ref="D62" location="'Country Stats'!A1" display="Country Stats" xr:uid="{37F97D7D-6476-49BF-9118-0DA3787A2751}"/>
+    <hyperlink ref="D10" r:id="rId1" xr:uid="{72FE398A-55A6-46EF-88FD-8804913A2E2A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
   <tableParts count="5">
-    <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
     <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5676,18 +5718,18 @@
       <c r="G2" s="76"/>
       <c r="H2" s="76"/>
     </row>
-    <row r="3" spans="1:8" ht="14.45" customHeight="1">
-      <c r="B3" s="84" t="str">
+    <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="B3" s="119" t="str">
         <f ca="1">HYPERLINK("#" &amp; CELL("address", _xlfn.XLOOKUP(Name,tbl_DfOverview[Dataframe],tbl_DfOverview[_],tbl_DfOverview[[#Headers],[_]])), "Overview ↩")</f>
         <v>Overview ↩</v>
       </c>
-      <c r="C3" s="84"/>
+      <c r="C3" s="83"/>
     </row>
     <row r="4" spans="1:8" ht="4.9000000000000004" customHeight="1">
       <c r="B4" s="69"/>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1">
-      <c r="B5" s="109" t="e" vm="1">
+      <c r="B5" s="108" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
       <c r="C5" s="78" t="s">
@@ -5698,14 +5740,14 @@
     <row r="6" spans="1:8" ht="10.15" customHeight="1"/>
     <row r="7" spans="1:8">
       <c r="A7" s="67"/>
-      <c r="B7" s="86" t="s">
+      <c r="B7" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="10.15" customHeight="1">
+    <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="67"/>
     </row>
     <row r="9" spans="1:8" ht="49.9" hidden="1" customHeight="1" outlineLevel="1">
@@ -5801,14 +5843,14 @@
     <row r="22" spans="1:6" ht="10.15" customHeight="1"/>
     <row r="23" spans="1:6" outlineLevel="1">
       <c r="A23" s="67"/>
-      <c r="B23" s="86" t="s">
+      <c r="B23" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="24" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A24" s="67"/>
     </row>
     <row r="25" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
@@ -5890,14 +5932,14 @@
     <row r="35" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
     <row r="36" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A36" s="67"/>
-      <c r="B36" s="86" t="s">
+      <c r="B36" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="37" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A37" s="67"/>
     </row>
     <row r="38" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
@@ -5952,14 +5994,14 @@
     <row r="45" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
     <row r="46" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A46" s="67"/>
-      <c r="B46" s="86" t="s">
+      <c r="B46" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="47" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A47" s="67"/>
     </row>
     <row r="48" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
@@ -6045,14 +6087,14 @@
     <row r="57" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
     <row r="58" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A58" s="67"/>
-      <c r="B58" s="86" t="s">
+      <c r="B58" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="59" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A59" s="67"/>
     </row>
     <row r="60" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">
@@ -6177,14 +6219,14 @@
     <row r="68" spans="1:6" ht="10.15" hidden="1" customHeight="1" outlineLevel="2"/>
     <row r="69" spans="1:6" outlineLevel="1" collapsed="1">
       <c r="A69" s="67"/>
-      <c r="B69" s="86" t="s">
+      <c r="B69" s="85" t="s">
         <v>61</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="10.15" customHeight="1" outlineLevel="1">
+    <row r="70" spans="1:6" ht="20.100000000000001" customHeight="1" outlineLevel="1">
       <c r="A70" s="67"/>
     </row>
     <row r="71" spans="1:6" ht="15" hidden="1" customHeight="1" outlineLevel="2">

</xml_diff>